<commit_message>
Se agregó qr a la plantilla excel y se mejoró el formato
</commit_message>
<xml_diff>
--- a/netlify/functions/plantilla.xlsx
+++ b/netlify/functions/plantilla.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL 2021\Documents\IGLESIA\sis presupuestos 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL 2021\Documents\IGLESIA\sis presupuestos 2\netlify\functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -20,132 +20,6 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>ejemplo:
-Barrio Colcapirua
-Rama Campoflores</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>notar:
-no colocar nada, 
-dato para el Sctrio. De Barrio</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K4" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>notas:
-Incluye: Sacerd, SocSoc, Niños&lt;8, ObMis, HistFam, EscD, Materiales de Escritorio.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K6" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>nota:
-Niños de 8 a11 años</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K9" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>nota:
-Colocar una X donde corresponda</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H11" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>notas:
-detallar la actividad</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J18" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Clases1:
-Marcar con X
-las que correspondan</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B21" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>nota:
-colocar encima correo electronico
-DEL Pte (a) o lider de la organizacion</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
@@ -1750,7 +1624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="150">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1965,67 +1839,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2041,20 +1877,70 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="45" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2067,16 +1953,16 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="45" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2115,44 +2001,61 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>280035</xdr:rowOff>
+      <xdr:colOff>178636</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>8466</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="714375" cy="714375"/>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>250371</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>24378</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="image1.jpg">
+        <xdr:cNvPr id="3" name="Imagen 2" descr="C:\Users\DELL 2021\Documents\IGLESIA\qr web sis presup.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
           </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="123825" y="3960495"/>
-          <a:ext cx="714375" cy="714375"/>
+          <a:off x="178636" y="3998080"/>
+          <a:ext cx="643235" cy="658169"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
         <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2452,7 +2355,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2479,21 +2382,20 @@
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="127" t="s">
+      <c r="C1" s="107" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
       <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="127"/>
-      <c r="I1" s="128"/>
+      <c r="H1" s="107"/>
+      <c r="I1" s="108"/>
       <c r="J1" s="4"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="129"/>
-      <c r="M1" s="112"/>
-      <c r="N1" s="112"/>
+      <c r="L1" s="109"/>
+      <c r="M1" s="100"/>
+      <c r="N1" s="100"/>
     </row>
     <row r="2" spans="1:14" ht="13.5" customHeight="1">
       <c r="A2" s="6"/>
@@ -2505,9 +2407,9 @@
         <v>3</v>
       </c>
       <c r="K2" s="8"/>
-      <c r="L2" s="130"/>
-      <c r="M2" s="131"/>
-      <c r="N2" s="131"/>
+      <c r="L2" s="110"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
     </row>
     <row r="3" spans="1:14" ht="13.5" customHeight="1">
       <c r="A3" s="9" t="s">
@@ -2518,10 +2420,10 @@
         <v>5</v>
       </c>
       <c r="L3" s="10"/>
-      <c r="M3" s="132" t="s">
+      <c r="M3" s="112" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="133"/>
+      <c r="N3" s="113"/>
     </row>
     <row r="4" spans="1:14" ht="13.5" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -2540,8 +2442,8 @@
         <v>8</v>
       </c>
       <c r="L4" s="13"/>
-      <c r="M4" s="134"/>
-      <c r="N4" s="135"/>
+      <c r="M4" s="114"/>
+      <c r="N4" s="115"/>
     </row>
     <row r="5" spans="1:14" ht="13.5" customHeight="1">
       <c r="A5" s="9" t="s">
@@ -2550,11 +2452,11 @@
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="114"/>
-      <c r="F5" s="112"/>
-      <c r="G5" s="112"/>
-      <c r="H5" s="112"/>
-      <c r="I5" s="112"/>
+      <c r="E5" s="99"/>
+      <c r="F5" s="100"/>
+      <c r="G5" s="100"/>
+      <c r="H5" s="100"/>
+      <c r="I5" s="100"/>
       <c r="J5" s="4"/>
       <c r="K5" s="14" t="s">
         <v>10</v>
@@ -2570,15 +2472,15 @@
         <v>12</v>
       </c>
       <c r="B6" s="9"/>
-      <c r="C6" s="111"/>
-      <c r="D6" s="112"/>
-      <c r="E6" s="112"/>
-      <c r="F6" s="112"/>
+      <c r="C6" s="120"/>
+      <c r="D6" s="100"/>
+      <c r="E6" s="100"/>
+      <c r="F6" s="100"/>
       <c r="G6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="113"/>
-      <c r="I6" s="99"/>
+      <c r="H6" s="121"/>
+      <c r="I6" s="119"/>
       <c r="J6" s="4"/>
       <c r="K6" s="14" t="s">
         <v>14</v>
@@ -2595,10 +2497,10 @@
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="114"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="D7" s="99"/>
+      <c r="E7" s="100"/>
+      <c r="F7" s="100"/>
+      <c r="G7" s="100"/>
       <c r="H7" s="9" t="s">
         <v>17</v>
       </c>
@@ -2607,8 +2509,8 @@
       <c r="K7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="115"/>
-      <c r="M7" s="116"/>
+      <c r="L7" s="122"/>
+      <c r="M7" s="123"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:14" ht="13.5" customHeight="1">
@@ -2626,19 +2528,19 @@
         <v>21</v>
       </c>
       <c r="K8" s="21"/>
-      <c r="L8" s="119"/>
-      <c r="M8" s="103"/>
-      <c r="N8" s="103"/>
+      <c r="L8" s="126"/>
+      <c r="M8" s="97"/>
+      <c r="N8" s="97"/>
     </row>
     <row r="9" spans="1:14" ht="13.5" customHeight="1">
       <c r="A9" s="94" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="114"/>
-      <c r="D9" s="112"/>
-      <c r="E9" s="112"/>
-      <c r="F9" s="112"/>
-      <c r="G9" s="112"/>
+      <c r="C9" s="99"/>
+      <c r="D9" s="100"/>
+      <c r="E9" s="100"/>
+      <c r="F9" s="100"/>
+      <c r="G9" s="100"/>
       <c r="J9" s="22" t="s">
         <v>68</v>
       </c>
@@ -2675,40 +2577,40 @@
       <c r="N11" s="28"/>
     </row>
     <row r="12" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A12" s="136"/>
-      <c r="B12" s="136"/>
-      <c r="C12" s="136"/>
-      <c r="D12" s="136"/>
-      <c r="E12" s="136"/>
-      <c r="F12" s="136"/>
-      <c r="G12" s="136"/>
-      <c r="H12" s="136"/>
-      <c r="I12" s="137"/>
+      <c r="A12" s="101"/>
+      <c r="B12" s="101"/>
+      <c r="C12" s="101"/>
+      <c r="D12" s="101"/>
+      <c r="E12" s="101"/>
+      <c r="F12" s="101"/>
+      <c r="G12" s="101"/>
+      <c r="H12" s="101"/>
+      <c r="I12" s="102"/>
       <c r="J12" s="27"/>
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A13" s="136"/>
-      <c r="B13" s="136"/>
-      <c r="C13" s="136"/>
-      <c r="D13" s="136"/>
-      <c r="E13" s="136"/>
-      <c r="F13" s="136"/>
-      <c r="G13" s="136"/>
-      <c r="H13" s="136"/>
-      <c r="I13" s="137"/>
+      <c r="A13" s="101"/>
+      <c r="B13" s="101"/>
+      <c r="C13" s="101"/>
+      <c r="D13" s="101"/>
+      <c r="E13" s="101"/>
+      <c r="F13" s="101"/>
+      <c r="G13" s="101"/>
+      <c r="H13" s="101"/>
+      <c r="I13" s="102"/>
       <c r="J13" s="11"/>
     </row>
     <row r="14" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A14" s="136"/>
-      <c r="B14" s="136"/>
-      <c r="C14" s="136"/>
-      <c r="D14" s="136"/>
-      <c r="E14" s="136"/>
-      <c r="F14" s="136"/>
-      <c r="G14" s="136"/>
-      <c r="H14" s="136"/>
-      <c r="I14" s="137"/>
+      <c r="A14" s="101"/>
+      <c r="B14" s="101"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="101"/>
+      <c r="E14" s="101"/>
+      <c r="F14" s="101"/>
+      <c r="G14" s="101"/>
+      <c r="H14" s="101"/>
+      <c r="I14" s="102"/>
       <c r="J14" s="29"/>
       <c r="K14" s="6"/>
       <c r="L14" s="30"/>
@@ -2716,15 +2618,15 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A15" s="136"/>
-      <c r="B15" s="136"/>
-      <c r="C15" s="136"/>
-      <c r="D15" s="136"/>
-      <c r="E15" s="136"/>
-      <c r="F15" s="136"/>
-      <c r="G15" s="136"/>
-      <c r="H15" s="136"/>
-      <c r="I15" s="137"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="101"/>
+      <c r="C15" s="101"/>
+      <c r="D15" s="101"/>
+      <c r="E15" s="101"/>
+      <c r="F15" s="101"/>
+      <c r="G15" s="101"/>
+      <c r="H15" s="101"/>
+      <c r="I15" s="102"/>
       <c r="J15" s="29" t="s">
         <v>27</v>
       </c>
@@ -2734,15 +2636,15 @@
       <c r="N15" s="28"/>
     </row>
     <row r="16" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A16" s="136"/>
-      <c r="B16" s="136"/>
-      <c r="C16" s="136"/>
-      <c r="D16" s="136"/>
-      <c r="E16" s="136"/>
-      <c r="F16" s="136"/>
-      <c r="G16" s="136"/>
-      <c r="H16" s="136"/>
-      <c r="I16" s="137"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="101"/>
+      <c r="C16" s="101"/>
+      <c r="D16" s="101"/>
+      <c r="E16" s="101"/>
+      <c r="F16" s="101"/>
+      <c r="G16" s="101"/>
+      <c r="H16" s="101"/>
+      <c r="I16" s="102"/>
       <c r="J16" s="33" t="s">
         <v>28</v>
       </c>
@@ -2750,21 +2652,21 @@
         <v>66</v>
       </c>
       <c r="L16" s="35"/>
-      <c r="M16" s="100" t="s">
+      <c r="M16" s="150" t="s">
         <v>67</v>
       </c>
-      <c r="N16" s="101"/>
+      <c r="N16" s="151"/>
     </row>
     <row r="17" spans="1:14" ht="14.4">
-      <c r="A17" s="136"/>
-      <c r="B17" s="136"/>
-      <c r="C17" s="136"/>
-      <c r="D17" s="136"/>
-      <c r="E17" s="136"/>
-      <c r="F17" s="136"/>
-      <c r="G17" s="136"/>
-      <c r="H17" s="136"/>
-      <c r="I17" s="137"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="101"/>
+      <c r="C17" s="101"/>
+      <c r="D17" s="101"/>
+      <c r="E17" s="101"/>
+      <c r="F17" s="101"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="101"/>
+      <c r="I17" s="102"/>
       <c r="J17" s="36" t="s">
         <v>29</v>
       </c>
@@ -2774,28 +2676,28 @@
         <v>30</v>
       </c>
       <c r="J18" s="38"/>
-      <c r="K18" s="102" t="s">
+      <c r="K18" s="124" t="s">
         <v>31</v>
       </c>
-      <c r="L18" s="103"/>
-      <c r="M18" s="103"/>
-      <c r="N18" s="104"/>
+      <c r="L18" s="97"/>
+      <c r="M18" s="97"/>
+      <c r="N18" s="98"/>
     </row>
     <row r="19" spans="1:14" ht="13.5" customHeight="1">
       <c r="J19" s="38"/>
-      <c r="K19" s="102" t="s">
+      <c r="K19" s="124" t="s">
         <v>32</v>
       </c>
-      <c r="L19" s="103"/>
-      <c r="M19" s="103"/>
-      <c r="N19" s="104"/>
+      <c r="L19" s="97"/>
+      <c r="M19" s="97"/>
+      <c r="N19" s="98"/>
     </row>
     <row r="20" spans="1:14" ht="13.5" customHeight="1">
-      <c r="B20" s="117"/>
-      <c r="C20" s="118"/>
-      <c r="D20" s="118"/>
-      <c r="E20" s="118"/>
-      <c r="F20" s="118"/>
+      <c r="B20" s="125"/>
+      <c r="C20" s="104"/>
+      <c r="D20" s="104"/>
+      <c r="E20" s="104"/>
+      <c r="F20" s="104"/>
       <c r="H20" s="39"/>
       <c r="J20" s="40"/>
       <c r="K20" s="41"/>
@@ -2810,59 +2712,59 @@
       <c r="D21" s="43"/>
       <c r="E21" s="26"/>
       <c r="J21" s="38"/>
-      <c r="K21" s="102" t="s">
+      <c r="K21" s="124" t="s">
         <v>34</v>
       </c>
-      <c r="L21" s="103"/>
-      <c r="M21" s="103"/>
-      <c r="N21" s="104"/>
+      <c r="L21" s="97"/>
+      <c r="M21" s="97"/>
+      <c r="N21" s="98"/>
     </row>
     <row r="22" spans="1:14" ht="23.25" customHeight="1">
       <c r="B22" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="140"/>
-      <c r="D22" s="140"/>
-      <c r="E22" s="140"/>
-      <c r="G22" s="138"/>
-      <c r="H22" s="118"/>
+      <c r="C22" s="106"/>
+      <c r="D22" s="106"/>
+      <c r="E22" s="106"/>
+      <c r="G22" s="152"/>
+      <c r="H22" s="153"/>
       <c r="J22" s="38"/>
-      <c r="K22" s="102" t="s">
+      <c r="K22" s="124" t="s">
         <v>36</v>
       </c>
-      <c r="L22" s="103"/>
-      <c r="M22" s="103"/>
-      <c r="N22" s="104"/>
+      <c r="L22" s="97"/>
+      <c r="M22" s="97"/>
+      <c r="N22" s="98"/>
     </row>
     <row r="23" spans="1:14" ht="17.25" customHeight="1">
       <c r="B23" s="44"/>
       <c r="C23" s="44"/>
-      <c r="D23" s="139" t="s">
+      <c r="D23" s="105" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="118"/>
-      <c r="F23" s="118"/>
-      <c r="G23" s="118"/>
-      <c r="H23" s="118"/>
-      <c r="I23" s="118"/>
+      <c r="E23" s="104"/>
+      <c r="F23" s="104"/>
+      <c r="G23" s="104"/>
+      <c r="H23" s="104"/>
+      <c r="I23" s="104"/>
       <c r="J23" s="38"/>
-      <c r="K23" s="105" t="s">
+      <c r="K23" s="137" t="s">
         <v>38</v>
       </c>
-      <c r="L23" s="103"/>
-      <c r="M23" s="103"/>
-      <c r="N23" s="104"/>
+      <c r="L23" s="97"/>
+      <c r="M23" s="97"/>
+      <c r="N23" s="98"/>
     </row>
     <row r="24" spans="1:14" ht="13.5" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="44"/>
       <c r="C24" s="44"/>
-      <c r="D24" s="118"/>
-      <c r="E24" s="118"/>
-      <c r="F24" s="118"/>
-      <c r="G24" s="118"/>
-      <c r="H24" s="118"/>
-      <c r="I24" s="118"/>
+      <c r="D24" s="104"/>
+      <c r="E24" s="104"/>
+      <c r="F24" s="104"/>
+      <c r="G24" s="104"/>
+      <c r="H24" s="104"/>
+      <c r="I24" s="104"/>
       <c r="J24" s="40"/>
       <c r="K24" s="41"/>
       <c r="L24" s="42"/>
@@ -2873,17 +2775,17 @@
       <c r="A25" s="44"/>
       <c r="B25" s="44"/>
       <c r="C25" s="44"/>
-      <c r="D25" s="118"/>
-      <c r="E25" s="118"/>
-      <c r="F25" s="118"/>
-      <c r="G25" s="118"/>
-      <c r="H25" s="118"/>
-      <c r="I25" s="118"/>
+      <c r="D25" s="104"/>
+      <c r="E25" s="104"/>
+      <c r="F25" s="104"/>
+      <c r="G25" s="104"/>
+      <c r="H25" s="104"/>
+      <c r="I25" s="104"/>
       <c r="J25" s="38"/>
-      <c r="K25" s="105"/>
-      <c r="L25" s="148"/>
-      <c r="M25" s="148"/>
-      <c r="N25" s="149"/>
+      <c r="K25" s="137"/>
+      <c r="L25" s="138"/>
+      <c r="M25" s="138"/>
+      <c r="N25" s="139"/>
     </row>
     <row r="26" spans="1:14" ht="13.5" customHeight="1">
       <c r="J26" s="38"/>
@@ -2932,218 +2834,218 @@
       <c r="L28" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="M28" s="107" t="s">
+      <c r="M28" s="140" t="s">
         <v>46</v>
       </c>
-      <c r="N28" s="108"/>
+      <c r="N28" s="141"/>
     </row>
     <row r="29" spans="1:14" ht="13.5" customHeight="1">
       <c r="A29" s="65"/>
-      <c r="B29" s="120"/>
-      <c r="C29" s="121"/>
-      <c r="D29" s="121"/>
-      <c r="E29" s="121"/>
-      <c r="F29" s="121"/>
-      <c r="G29" s="121"/>
-      <c r="H29" s="121"/>
-      <c r="I29" s="122"/>
+      <c r="B29" s="127"/>
+      <c r="C29" s="128"/>
+      <c r="D29" s="128"/>
+      <c r="E29" s="128"/>
+      <c r="F29" s="128"/>
+      <c r="G29" s="128"/>
+      <c r="H29" s="128"/>
+      <c r="I29" s="129"/>
       <c r="J29" s="66"/>
       <c r="K29" s="67"/>
       <c r="L29" s="68"/>
-      <c r="M29" s="96"/>
-      <c r="N29" s="97"/>
+      <c r="M29" s="133"/>
+      <c r="N29" s="134"/>
     </row>
     <row r="30" spans="1:14" ht="13.5" customHeight="1">
       <c r="A30" s="69"/>
-      <c r="B30" s="123"/>
-      <c r="C30" s="103"/>
-      <c r="D30" s="103"/>
-      <c r="E30" s="103"/>
-      <c r="F30" s="103"/>
-      <c r="G30" s="103"/>
-      <c r="H30" s="103"/>
-      <c r="I30" s="104"/>
+      <c r="B30" s="96"/>
+      <c r="C30" s="97"/>
+      <c r="D30" s="97"/>
+      <c r="E30" s="97"/>
+      <c r="F30" s="97"/>
+      <c r="G30" s="97"/>
+      <c r="H30" s="97"/>
+      <c r="I30" s="98"/>
       <c r="J30" s="70"/>
       <c r="K30" s="71"/>
       <c r="L30" s="72"/>
-      <c r="M30" s="98"/>
-      <c r="N30" s="99"/>
+      <c r="M30" s="118"/>
+      <c r="N30" s="119"/>
     </row>
     <row r="31" spans="1:14" ht="13.5" customHeight="1">
       <c r="A31" s="69"/>
-      <c r="B31" s="123"/>
-      <c r="C31" s="103"/>
-      <c r="D31" s="103"/>
-      <c r="E31" s="103"/>
-      <c r="F31" s="103"/>
-      <c r="G31" s="103"/>
-      <c r="H31" s="103"/>
-      <c r="I31" s="104"/>
+      <c r="B31" s="96"/>
+      <c r="C31" s="97"/>
+      <c r="D31" s="97"/>
+      <c r="E31" s="97"/>
+      <c r="F31" s="97"/>
+      <c r="G31" s="97"/>
+      <c r="H31" s="97"/>
+      <c r="I31" s="98"/>
       <c r="J31" s="73"/>
       <c r="K31" s="71"/>
       <c r="L31" s="72"/>
-      <c r="M31" s="98"/>
-      <c r="N31" s="99"/>
+      <c r="M31" s="118"/>
+      <c r="N31" s="119"/>
     </row>
     <row r="32" spans="1:14" ht="13.5" customHeight="1">
       <c r="A32" s="69"/>
-      <c r="B32" s="123"/>
-      <c r="C32" s="103"/>
-      <c r="D32" s="103"/>
-      <c r="E32" s="103"/>
-      <c r="F32" s="103"/>
-      <c r="G32" s="103"/>
-      <c r="H32" s="103"/>
-      <c r="I32" s="104"/>
+      <c r="B32" s="96"/>
+      <c r="C32" s="97"/>
+      <c r="D32" s="97"/>
+      <c r="E32" s="97"/>
+      <c r="F32" s="97"/>
+      <c r="G32" s="97"/>
+      <c r="H32" s="97"/>
+      <c r="I32" s="98"/>
       <c r="J32" s="73"/>
       <c r="K32" s="71"/>
       <c r="L32" s="72"/>
-      <c r="M32" s="98"/>
-      <c r="N32" s="99"/>
+      <c r="M32" s="118"/>
+      <c r="N32" s="119"/>
     </row>
     <row r="33" spans="1:14" ht="13.5" customHeight="1">
       <c r="A33" s="69"/>
-      <c r="B33" s="123"/>
-      <c r="C33" s="103"/>
-      <c r="D33" s="103"/>
-      <c r="E33" s="103"/>
-      <c r="F33" s="103"/>
-      <c r="G33" s="103"/>
-      <c r="H33" s="103"/>
-      <c r="I33" s="104"/>
+      <c r="B33" s="96"/>
+      <c r="C33" s="97"/>
+      <c r="D33" s="97"/>
+      <c r="E33" s="97"/>
+      <c r="F33" s="97"/>
+      <c r="G33" s="97"/>
+      <c r="H33" s="97"/>
+      <c r="I33" s="98"/>
       <c r="J33" s="73"/>
       <c r="K33" s="71"/>
       <c r="L33" s="72"/>
-      <c r="M33" s="98"/>
-      <c r="N33" s="99"/>
+      <c r="M33" s="118"/>
+      <c r="N33" s="119"/>
     </row>
     <row r="34" spans="1:14" ht="13.5" customHeight="1">
       <c r="A34" s="69"/>
-      <c r="B34" s="123"/>
-      <c r="C34" s="103"/>
-      <c r="D34" s="103"/>
-      <c r="E34" s="103"/>
-      <c r="F34" s="103"/>
-      <c r="G34" s="103"/>
-      <c r="H34" s="103"/>
-      <c r="I34" s="104"/>
+      <c r="B34" s="96"/>
+      <c r="C34" s="97"/>
+      <c r="D34" s="97"/>
+      <c r="E34" s="97"/>
+      <c r="F34" s="97"/>
+      <c r="G34" s="97"/>
+      <c r="H34" s="97"/>
+      <c r="I34" s="98"/>
       <c r="J34" s="70"/>
       <c r="K34" s="71"/>
       <c r="L34" s="72"/>
-      <c r="M34" s="98"/>
-      <c r="N34" s="99"/>
+      <c r="M34" s="118"/>
+      <c r="N34" s="119"/>
     </row>
     <row r="35" spans="1:14" ht="13.5" customHeight="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="123"/>
-      <c r="C35" s="103"/>
-      <c r="D35" s="103"/>
-      <c r="E35" s="103"/>
-      <c r="F35" s="103"/>
-      <c r="G35" s="103"/>
-      <c r="H35" s="103"/>
-      <c r="I35" s="104"/>
+      <c r="B35" s="96"/>
+      <c r="C35" s="97"/>
+      <c r="D35" s="97"/>
+      <c r="E35" s="97"/>
+      <c r="F35" s="97"/>
+      <c r="G35" s="97"/>
+      <c r="H35" s="97"/>
+      <c r="I35" s="98"/>
       <c r="J35" s="70"/>
       <c r="K35" s="71"/>
       <c r="L35" s="72"/>
-      <c r="M35" s="98"/>
-      <c r="N35" s="99"/>
+      <c r="M35" s="118"/>
+      <c r="N35" s="119"/>
     </row>
     <row r="36" spans="1:14" ht="13.5" customHeight="1">
       <c r="A36" s="69"/>
-      <c r="B36" s="123"/>
-      <c r="C36" s="103"/>
-      <c r="D36" s="103"/>
-      <c r="E36" s="103"/>
-      <c r="F36" s="103"/>
-      <c r="G36" s="103"/>
-      <c r="H36" s="103"/>
-      <c r="I36" s="104"/>
+      <c r="B36" s="96"/>
+      <c r="C36" s="97"/>
+      <c r="D36" s="97"/>
+      <c r="E36" s="97"/>
+      <c r="F36" s="97"/>
+      <c r="G36" s="97"/>
+      <c r="H36" s="97"/>
+      <c r="I36" s="98"/>
       <c r="J36" s="70"/>
       <c r="K36" s="71"/>
       <c r="L36" s="72"/>
-      <c r="M36" s="98"/>
-      <c r="N36" s="99"/>
+      <c r="M36" s="118"/>
+      <c r="N36" s="119"/>
     </row>
     <row r="37" spans="1:14" ht="13.5" customHeight="1">
       <c r="A37" s="69"/>
-      <c r="B37" s="123"/>
-      <c r="C37" s="103"/>
-      <c r="D37" s="103"/>
-      <c r="E37" s="103"/>
-      <c r="F37" s="103"/>
-      <c r="G37" s="103"/>
-      <c r="H37" s="103"/>
-      <c r="I37" s="104"/>
+      <c r="B37" s="96"/>
+      <c r="C37" s="97"/>
+      <c r="D37" s="97"/>
+      <c r="E37" s="97"/>
+      <c r="F37" s="97"/>
+      <c r="G37" s="97"/>
+      <c r="H37" s="97"/>
+      <c r="I37" s="98"/>
       <c r="J37" s="70"/>
       <c r="K37" s="71"/>
       <c r="L37" s="72"/>
-      <c r="M37" s="98"/>
-      <c r="N37" s="99"/>
+      <c r="M37" s="118"/>
+      <c r="N37" s="119"/>
     </row>
     <row r="38" spans="1:14" ht="13.5" customHeight="1">
       <c r="A38" s="69"/>
-      <c r="B38" s="123"/>
-      <c r="C38" s="103"/>
-      <c r="D38" s="103"/>
-      <c r="E38" s="103"/>
-      <c r="F38" s="103"/>
-      <c r="G38" s="103"/>
-      <c r="H38" s="103"/>
-      <c r="I38" s="104"/>
+      <c r="B38" s="96"/>
+      <c r="C38" s="97"/>
+      <c r="D38" s="97"/>
+      <c r="E38" s="97"/>
+      <c r="F38" s="97"/>
+      <c r="G38" s="97"/>
+      <c r="H38" s="97"/>
+      <c r="I38" s="98"/>
       <c r="J38" s="70"/>
       <c r="K38" s="71"/>
       <c r="L38" s="72"/>
-      <c r="M38" s="98"/>
-      <c r="N38" s="99"/>
+      <c r="M38" s="118"/>
+      <c r="N38" s="119"/>
     </row>
     <row r="39" spans="1:14" ht="13.5" customHeight="1">
       <c r="A39" s="69"/>
-      <c r="B39" s="123"/>
-      <c r="C39" s="103"/>
-      <c r="D39" s="103"/>
-      <c r="E39" s="103"/>
-      <c r="F39" s="103"/>
-      <c r="G39" s="103"/>
-      <c r="H39" s="103"/>
-      <c r="I39" s="104"/>
+      <c r="B39" s="96"/>
+      <c r="C39" s="97"/>
+      <c r="D39" s="97"/>
+      <c r="E39" s="97"/>
+      <c r="F39" s="97"/>
+      <c r="G39" s="97"/>
+      <c r="H39" s="97"/>
+      <c r="I39" s="98"/>
       <c r="J39" s="70"/>
       <c r="K39" s="71"/>
       <c r="L39" s="72"/>
-      <c r="M39" s="98"/>
-      <c r="N39" s="99"/>
+      <c r="M39" s="118"/>
+      <c r="N39" s="119"/>
     </row>
     <row r="40" spans="1:14" ht="13.5" customHeight="1">
       <c r="A40" s="69"/>
-      <c r="B40" s="123"/>
-      <c r="C40" s="103"/>
-      <c r="D40" s="103"/>
-      <c r="E40" s="103"/>
-      <c r="F40" s="103"/>
-      <c r="G40" s="103"/>
-      <c r="H40" s="103"/>
-      <c r="I40" s="104"/>
+      <c r="B40" s="96"/>
+      <c r="C40" s="97"/>
+      <c r="D40" s="97"/>
+      <c r="E40" s="97"/>
+      <c r="F40" s="97"/>
+      <c r="G40" s="97"/>
+      <c r="H40" s="97"/>
+      <c r="I40" s="98"/>
       <c r="J40" s="70"/>
       <c r="K40" s="71"/>
       <c r="L40" s="72"/>
-      <c r="M40" s="98"/>
-      <c r="N40" s="99"/>
+      <c r="M40" s="118"/>
+      <c r="N40" s="119"/>
     </row>
     <row r="41" spans="1:14" ht="13.5" customHeight="1">
       <c r="A41" s="74"/>
-      <c r="B41" s="124"/>
-      <c r="C41" s="125"/>
-      <c r="D41" s="125"/>
-      <c r="E41" s="125"/>
-      <c r="F41" s="125"/>
-      <c r="G41" s="125"/>
-      <c r="H41" s="125"/>
-      <c r="I41" s="126"/>
+      <c r="B41" s="130"/>
+      <c r="C41" s="131"/>
+      <c r="D41" s="131"/>
+      <c r="E41" s="131"/>
+      <c r="F41" s="131"/>
+      <c r="G41" s="131"/>
+      <c r="H41" s="131"/>
+      <c r="I41" s="132"/>
       <c r="J41" s="75"/>
       <c r="K41" s="76"/>
       <c r="L41" s="77"/>
-      <c r="M41" s="109"/>
-      <c r="N41" s="110"/>
+      <c r="M41" s="116"/>
+      <c r="N41" s="117"/>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
       <c r="A42" s="78"/>
@@ -3243,24 +3145,23 @@
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A12:I17"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="D23:I25"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="M3:N4"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="K18:N18"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="K22:N22"/>
+    <mergeCell ref="K23:N23"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="M37:N37"/>
     <mergeCell ref="M41:N41"/>
     <mergeCell ref="M40:N40"/>
     <mergeCell ref="C6:F6"/>
@@ -3277,23 +3178,24 @@
     <mergeCell ref="B38:I38"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B41:I41"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="M37:N37"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="K18:N18"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="K22:N22"/>
-    <mergeCell ref="K23:N23"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="M3:N4"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A12:I17"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="D23:I25"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B36:I36"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:E1 H1:I1 L2:N2 E5:I5 C6:F6 H6:I6 D7:G7 B8 L8 A12:I17 K16 M16:N16 B20:F20 C22 G22:H22">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
@@ -3312,7 +3214,6 @@
     <oddFooter>&amp;R00-024βэηяμ</oddFooter>
   </headerFooter>
   <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -3340,21 +3241,21 @@
         <v>54</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
+      <c r="C1" s="107"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
       <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="127"/>
-      <c r="I1" s="128"/>
+      <c r="H1" s="107"/>
+      <c r="I1" s="108"/>
       <c r="J1" s="4"/>
       <c r="K1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="129"/>
-      <c r="M1" s="112"/>
-      <c r="N1" s="112"/>
+      <c r="L1" s="109"/>
+      <c r="M1" s="100"/>
+      <c r="N1" s="100"/>
     </row>
     <row r="2" spans="1:14" ht="13.5" customHeight="1">
       <c r="A2" s="6"/>
@@ -3366,9 +3267,9 @@
         <v>3</v>
       </c>
       <c r="K2" s="8"/>
-      <c r="L2" s="147"/>
-      <c r="M2" s="103"/>
-      <c r="N2" s="103"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
     </row>
     <row r="3" spans="1:14" ht="13.5" customHeight="1">
       <c r="A3" s="9" t="s">
@@ -3379,10 +3280,10 @@
         <v>5</v>
       </c>
       <c r="L3" s="10"/>
-      <c r="M3" s="132" t="s">
+      <c r="M3" s="112" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="133"/>
+      <c r="N3" s="113"/>
     </row>
     <row r="4" spans="1:14" ht="13.5" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -3401,8 +3302,8 @@
         <v>8</v>
       </c>
       <c r="L4" s="13"/>
-      <c r="M4" s="134"/>
-      <c r="N4" s="135"/>
+      <c r="M4" s="114"/>
+      <c r="N4" s="115"/>
     </row>
     <row r="5" spans="1:14" ht="13.5" customHeight="1">
       <c r="A5" s="9" t="s">
@@ -3411,11 +3312,11 @@
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="114"/>
-      <c r="F5" s="112"/>
-      <c r="G5" s="112"/>
-      <c r="H5" s="112"/>
-      <c r="I5" s="112"/>
+      <c r="E5" s="99"/>
+      <c r="F5" s="100"/>
+      <c r="G5" s="100"/>
+      <c r="H5" s="100"/>
+      <c r="I5" s="100"/>
       <c r="J5" s="4"/>
       <c r="K5" s="14" t="s">
         <v>10</v>
@@ -3431,15 +3332,15 @@
         <v>12</v>
       </c>
       <c r="B6" s="9"/>
-      <c r="C6" s="111"/>
-      <c r="D6" s="112"/>
-      <c r="E6" s="112"/>
-      <c r="F6" s="112"/>
+      <c r="C6" s="120"/>
+      <c r="D6" s="100"/>
+      <c r="E6" s="100"/>
+      <c r="F6" s="100"/>
       <c r="G6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="113"/>
-      <c r="I6" s="99"/>
+      <c r="H6" s="121"/>
+      <c r="I6" s="119"/>
       <c r="J6" s="4"/>
       <c r="K6" s="14" t="s">
         <v>14</v>
@@ -3456,10 +3357,10 @@
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="114"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="D7" s="99"/>
+      <c r="E7" s="100"/>
+      <c r="F7" s="100"/>
+      <c r="G7" s="100"/>
       <c r="H7" s="9" t="s">
         <v>17</v>
       </c>
@@ -3468,11 +3369,11 @@
       <c r="K7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="146">
+      <c r="L7" s="143">
         <f>SUM(L4:L6)+N5+N6</f>
         <v>0</v>
       </c>
-      <c r="M7" s="116"/>
+      <c r="M7" s="123"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:14" ht="13.5" customHeight="1">
@@ -3490,22 +3391,22 @@
         <v>21</v>
       </c>
       <c r="K8" s="21"/>
-      <c r="L8" s="119"/>
-      <c r="M8" s="103"/>
-      <c r="N8" s="103"/>
+      <c r="L8" s="126"/>
+      <c r="M8" s="97"/>
+      <c r="N8" s="97"/>
     </row>
     <row r="9" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A9" s="144" t="s">
+      <c r="A9" s="148" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="118"/>
-      <c r="C9" s="118"/>
-      <c r="D9" s="118"/>
-      <c r="E9" s="118"/>
-      <c r="F9" s="118"/>
-      <c r="G9" s="118"/>
-      <c r="H9" s="118"/>
-      <c r="I9" s="145"/>
+      <c r="B9" s="104"/>
+      <c r="C9" s="104"/>
+      <c r="D9" s="104"/>
+      <c r="E9" s="104"/>
+      <c r="F9" s="104"/>
+      <c r="G9" s="104"/>
+      <c r="H9" s="104"/>
+      <c r="I9" s="149"/>
       <c r="J9" s="22" t="s">
         <v>23</v>
       </c>
@@ -3540,40 +3441,40 @@
       <c r="N11" s="28"/>
     </row>
     <row r="12" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A12" s="141"/>
-      <c r="B12" s="112"/>
-      <c r="C12" s="112"/>
-      <c r="D12" s="112"/>
-      <c r="E12" s="112"/>
-      <c r="F12" s="112"/>
-      <c r="G12" s="112"/>
-      <c r="H12" s="112"/>
-      <c r="I12" s="128"/>
+      <c r="A12" s="145"/>
+      <c r="B12" s="100"/>
+      <c r="C12" s="100"/>
+      <c r="D12" s="100"/>
+      <c r="E12" s="100"/>
+      <c r="F12" s="100"/>
+      <c r="G12" s="100"/>
+      <c r="H12" s="100"/>
+      <c r="I12" s="108"/>
       <c r="J12" s="27"/>
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A13" s="142"/>
-      <c r="B13" s="103"/>
-      <c r="C13" s="103"/>
-      <c r="D13" s="103"/>
-      <c r="E13" s="103"/>
-      <c r="F13" s="103"/>
-      <c r="G13" s="103"/>
-      <c r="H13" s="103"/>
-      <c r="I13" s="99"/>
+      <c r="A13" s="146"/>
+      <c r="B13" s="97"/>
+      <c r="C13" s="97"/>
+      <c r="D13" s="97"/>
+      <c r="E13" s="97"/>
+      <c r="F13" s="97"/>
+      <c r="G13" s="97"/>
+      <c r="H13" s="97"/>
+      <c r="I13" s="119"/>
       <c r="J13" s="11"/>
     </row>
     <row r="14" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A14" s="142"/>
-      <c r="B14" s="103"/>
-      <c r="C14" s="103"/>
-      <c r="D14" s="103"/>
-      <c r="E14" s="103"/>
-      <c r="F14" s="103"/>
-      <c r="G14" s="103"/>
-      <c r="H14" s="103"/>
-      <c r="I14" s="99"/>
+      <c r="A14" s="146"/>
+      <c r="B14" s="97"/>
+      <c r="C14" s="97"/>
+      <c r="D14" s="97"/>
+      <c r="E14" s="97"/>
+      <c r="F14" s="97"/>
+      <c r="G14" s="97"/>
+      <c r="H14" s="97"/>
+      <c r="I14" s="119"/>
       <c r="J14" s="29"/>
       <c r="K14" s="6"/>
       <c r="L14" s="30"/>
@@ -3581,15 +3482,15 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A15" s="142"/>
-      <c r="B15" s="103"/>
-      <c r="C15" s="103"/>
-      <c r="D15" s="103"/>
-      <c r="E15" s="103"/>
-      <c r="F15" s="103"/>
-      <c r="G15" s="103"/>
-      <c r="H15" s="103"/>
-      <c r="I15" s="99"/>
+      <c r="A15" s="146"/>
+      <c r="B15" s="97"/>
+      <c r="C15" s="97"/>
+      <c r="D15" s="97"/>
+      <c r="E15" s="97"/>
+      <c r="F15" s="97"/>
+      <c r="G15" s="97"/>
+      <c r="H15" s="97"/>
+      <c r="I15" s="119"/>
       <c r="J15" s="29" t="s">
         <v>55</v>
       </c>
@@ -3600,33 +3501,33 @@
       <c r="N15" s="28"/>
     </row>
     <row r="16" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A16" s="142"/>
-      <c r="B16" s="103"/>
-      <c r="C16" s="103"/>
-      <c r="D16" s="103"/>
-      <c r="E16" s="103"/>
-      <c r="F16" s="103"/>
-      <c r="G16" s="103"/>
-      <c r="H16" s="103"/>
-      <c r="I16" s="99"/>
+      <c r="A16" s="146"/>
+      <c r="B16" s="97"/>
+      <c r="C16" s="97"/>
+      <c r="D16" s="97"/>
+      <c r="E16" s="97"/>
+      <c r="F16" s="97"/>
+      <c r="G16" s="97"/>
+      <c r="H16" s="97"/>
+      <c r="I16" s="119"/>
       <c r="J16" s="33" t="s">
         <v>28</v>
       </c>
       <c r="K16" s="34"/>
       <c r="L16" s="35"/>
-      <c r="M16" s="100"/>
-      <c r="N16" s="101"/>
+      <c r="M16" s="135"/>
+      <c r="N16" s="136"/>
     </row>
     <row r="17" spans="1:14" ht="14.4">
-      <c r="A17" s="143"/>
-      <c r="B17" s="118"/>
-      <c r="C17" s="118"/>
-      <c r="D17" s="118"/>
-      <c r="E17" s="118"/>
-      <c r="F17" s="118"/>
-      <c r="G17" s="118"/>
-      <c r="H17" s="118"/>
-      <c r="I17" s="118"/>
+      <c r="A17" s="147"/>
+      <c r="B17" s="104"/>
+      <c r="C17" s="104"/>
+      <c r="D17" s="104"/>
+      <c r="E17" s="104"/>
+      <c r="F17" s="104"/>
+      <c r="G17" s="104"/>
+      <c r="H17" s="104"/>
+      <c r="I17" s="104"/>
       <c r="J17" s="36" t="s">
         <v>29</v>
       </c>
@@ -3636,28 +3537,28 @@
         <v>30</v>
       </c>
       <c r="J18" s="38"/>
-      <c r="K18" s="106" t="s">
+      <c r="K18" s="144" t="s">
         <v>57</v>
       </c>
-      <c r="L18" s="103"/>
-      <c r="M18" s="103"/>
-      <c r="N18" s="104"/>
+      <c r="L18" s="97"/>
+      <c r="M18" s="97"/>
+      <c r="N18" s="98"/>
     </row>
     <row r="19" spans="1:14" ht="13.5" customHeight="1">
       <c r="J19" s="38"/>
-      <c r="K19" s="106" t="s">
+      <c r="K19" s="144" t="s">
         <v>58</v>
       </c>
-      <c r="L19" s="103"/>
-      <c r="M19" s="103"/>
-      <c r="N19" s="104"/>
+      <c r="L19" s="97"/>
+      <c r="M19" s="97"/>
+      <c r="N19" s="98"/>
     </row>
     <row r="20" spans="1:14" ht="13.5" customHeight="1">
-      <c r="B20" s="117"/>
-      <c r="C20" s="118"/>
-      <c r="D20" s="118"/>
-      <c r="E20" s="118"/>
-      <c r="F20" s="118"/>
+      <c r="B20" s="125"/>
+      <c r="C20" s="104"/>
+      <c r="D20" s="104"/>
+      <c r="E20" s="104"/>
+      <c r="F20" s="104"/>
       <c r="H20" s="39"/>
       <c r="J20" s="40"/>
       <c r="K20" s="41" t="s">
@@ -3674,59 +3575,59 @@
       <c r="D21" s="43"/>
       <c r="E21" s="26"/>
       <c r="J21" s="38"/>
-      <c r="K21" s="106" t="s">
+      <c r="K21" s="144" t="s">
         <v>60</v>
       </c>
-      <c r="L21" s="103"/>
-      <c r="M21" s="103"/>
-      <c r="N21" s="104"/>
+      <c r="L21" s="97"/>
+      <c r="M21" s="97"/>
+      <c r="N21" s="98"/>
     </row>
     <row r="22" spans="1:14" ht="17.25" customHeight="1">
       <c r="C22" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D22" s="140"/>
-      <c r="E22" s="118"/>
+      <c r="D22" s="106"/>
+      <c r="E22" s="104"/>
       <c r="F22" s="26"/>
-      <c r="G22" s="138"/>
-      <c r="H22" s="118"/>
+      <c r="G22" s="103"/>
+      <c r="H22" s="104"/>
       <c r="J22" s="38"/>
-      <c r="K22" s="106" t="s">
+      <c r="K22" s="144" t="s">
         <v>61</v>
       </c>
-      <c r="L22" s="103"/>
-      <c r="M22" s="103"/>
-      <c r="N22" s="104"/>
+      <c r="L22" s="97"/>
+      <c r="M22" s="97"/>
+      <c r="N22" s="98"/>
     </row>
     <row r="23" spans="1:14" ht="17.25" customHeight="1">
       <c r="B23" s="44"/>
       <c r="C23" s="44"/>
-      <c r="D23" s="139" t="s">
+      <c r="D23" s="105" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="118"/>
-      <c r="F23" s="118"/>
-      <c r="G23" s="118"/>
-      <c r="H23" s="118"/>
-      <c r="I23" s="118"/>
+      <c r="E23" s="104"/>
+      <c r="F23" s="104"/>
+      <c r="G23" s="104"/>
+      <c r="H23" s="104"/>
+      <c r="I23" s="104"/>
       <c r="J23" s="38"/>
-      <c r="K23" s="106" t="s">
+      <c r="K23" s="144" t="s">
         <v>62</v>
       </c>
-      <c r="L23" s="103"/>
-      <c r="M23" s="103"/>
-      <c r="N23" s="104"/>
+      <c r="L23" s="97"/>
+      <c r="M23" s="97"/>
+      <c r="N23" s="98"/>
     </row>
     <row r="24" spans="1:14" ht="13.5" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="44"/>
       <c r="C24" s="44"/>
-      <c r="D24" s="118"/>
-      <c r="E24" s="118"/>
-      <c r="F24" s="118"/>
-      <c r="G24" s="118"/>
-      <c r="H24" s="118"/>
-      <c r="I24" s="118"/>
+      <c r="D24" s="104"/>
+      <c r="E24" s="104"/>
+      <c r="F24" s="104"/>
+      <c r="G24" s="104"/>
+      <c r="H24" s="104"/>
+      <c r="I24" s="104"/>
       <c r="J24" s="40"/>
       <c r="K24" s="41" t="s">
         <v>63</v>
@@ -3739,19 +3640,19 @@
       <c r="A25" s="44"/>
       <c r="B25" s="44"/>
       <c r="C25" s="44"/>
-      <c r="D25" s="118"/>
-      <c r="E25" s="118"/>
-      <c r="F25" s="118"/>
-      <c r="G25" s="118"/>
-      <c r="H25" s="118"/>
-      <c r="I25" s="118"/>
+      <c r="D25" s="104"/>
+      <c r="E25" s="104"/>
+      <c r="F25" s="104"/>
+      <c r="G25" s="104"/>
+      <c r="H25" s="104"/>
+      <c r="I25" s="104"/>
       <c r="J25" s="38"/>
-      <c r="K25" s="106" t="s">
+      <c r="K25" s="144" t="s">
         <v>64</v>
       </c>
-      <c r="L25" s="103"/>
-      <c r="M25" s="103"/>
-      <c r="N25" s="104"/>
+      <c r="L25" s="97"/>
+      <c r="M25" s="97"/>
+      <c r="N25" s="98"/>
     </row>
     <row r="26" spans="1:14" ht="13.5" customHeight="1">
       <c r="J26" s="38"/>
@@ -3802,257 +3703,257 @@
       <c r="L28" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="M28" s="107" t="s">
+      <c r="M28" s="140" t="s">
         <v>46</v>
       </c>
-      <c r="N28" s="108"/>
+      <c r="N28" s="141"/>
     </row>
     <row r="29" spans="1:14" ht="13.5" customHeight="1">
       <c r="A29" s="65"/>
-      <c r="B29" s="120"/>
-      <c r="C29" s="121"/>
-      <c r="D29" s="121"/>
-      <c r="E29" s="121"/>
-      <c r="F29" s="121"/>
-      <c r="G29" s="121"/>
-      <c r="H29" s="121"/>
-      <c r="I29" s="122"/>
+      <c r="B29" s="127"/>
+      <c r="C29" s="128"/>
+      <c r="D29" s="128"/>
+      <c r="E29" s="128"/>
+      <c r="F29" s="128"/>
+      <c r="G29" s="128"/>
+      <c r="H29" s="128"/>
+      <c r="I29" s="129"/>
       <c r="J29" s="66"/>
       <c r="K29" s="67">
         <f t="shared" ref="K29:K41" si="0">A29*J29</f>
         <v>0</v>
       </c>
       <c r="L29" s="68"/>
-      <c r="M29" s="96"/>
-      <c r="N29" s="97"/>
+      <c r="M29" s="133"/>
+      <c r="N29" s="134"/>
     </row>
     <row r="30" spans="1:14" ht="13.5" customHeight="1">
       <c r="A30" s="69"/>
-      <c r="B30" s="123"/>
-      <c r="C30" s="103"/>
-      <c r="D30" s="103"/>
-      <c r="E30" s="103"/>
-      <c r="F30" s="103"/>
-      <c r="G30" s="103"/>
-      <c r="H30" s="103"/>
-      <c r="I30" s="104"/>
+      <c r="B30" s="96"/>
+      <c r="C30" s="97"/>
+      <c r="D30" s="97"/>
+      <c r="E30" s="97"/>
+      <c r="F30" s="97"/>
+      <c r="G30" s="97"/>
+      <c r="H30" s="97"/>
+      <c r="I30" s="98"/>
       <c r="J30" s="70"/>
       <c r="K30" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L30" s="72"/>
-      <c r="M30" s="98"/>
-      <c r="N30" s="99"/>
+      <c r="M30" s="118"/>
+      <c r="N30" s="119"/>
     </row>
     <row r="31" spans="1:14" ht="13.5" customHeight="1">
       <c r="A31" s="69"/>
-      <c r="B31" s="123"/>
-      <c r="C31" s="103"/>
-      <c r="D31" s="103"/>
-      <c r="E31" s="103"/>
-      <c r="F31" s="103"/>
-      <c r="G31" s="103"/>
-      <c r="H31" s="103"/>
-      <c r="I31" s="104"/>
+      <c r="B31" s="96"/>
+      <c r="C31" s="97"/>
+      <c r="D31" s="97"/>
+      <c r="E31" s="97"/>
+      <c r="F31" s="97"/>
+      <c r="G31" s="97"/>
+      <c r="H31" s="97"/>
+      <c r="I31" s="98"/>
       <c r="J31" s="73"/>
       <c r="K31" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L31" s="72"/>
-      <c r="M31" s="98"/>
-      <c r="N31" s="99"/>
+      <c r="M31" s="118"/>
+      <c r="N31" s="119"/>
     </row>
     <row r="32" spans="1:14" ht="13.5" customHeight="1">
       <c r="A32" s="69"/>
-      <c r="B32" s="123"/>
-      <c r="C32" s="103"/>
-      <c r="D32" s="103"/>
-      <c r="E32" s="103"/>
-      <c r="F32" s="103"/>
-      <c r="G32" s="103"/>
-      <c r="H32" s="103"/>
-      <c r="I32" s="104"/>
+      <c r="B32" s="96"/>
+      <c r="C32" s="97"/>
+      <c r="D32" s="97"/>
+      <c r="E32" s="97"/>
+      <c r="F32" s="97"/>
+      <c r="G32" s="97"/>
+      <c r="H32" s="97"/>
+      <c r="I32" s="98"/>
       <c r="J32" s="73"/>
       <c r="K32" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L32" s="72"/>
-      <c r="M32" s="98"/>
-      <c r="N32" s="99"/>
+      <c r="M32" s="118"/>
+      <c r="N32" s="119"/>
     </row>
     <row r="33" spans="1:14" ht="13.5" customHeight="1">
       <c r="A33" s="69"/>
-      <c r="B33" s="123"/>
-      <c r="C33" s="103"/>
-      <c r="D33" s="103"/>
-      <c r="E33" s="103"/>
-      <c r="F33" s="103"/>
-      <c r="G33" s="103"/>
-      <c r="H33" s="103"/>
-      <c r="I33" s="104"/>
+      <c r="B33" s="96"/>
+      <c r="C33" s="97"/>
+      <c r="D33" s="97"/>
+      <c r="E33" s="97"/>
+      <c r="F33" s="97"/>
+      <c r="G33" s="97"/>
+      <c r="H33" s="97"/>
+      <c r="I33" s="98"/>
       <c r="J33" s="73"/>
       <c r="K33" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L33" s="72"/>
-      <c r="M33" s="98"/>
-      <c r="N33" s="99"/>
+      <c r="M33" s="118"/>
+      <c r="N33" s="119"/>
     </row>
     <row r="34" spans="1:14" ht="13.5" customHeight="1">
       <c r="A34" s="69"/>
-      <c r="B34" s="123"/>
-      <c r="C34" s="103"/>
-      <c r="D34" s="103"/>
-      <c r="E34" s="103"/>
-      <c r="F34" s="103"/>
-      <c r="G34" s="103"/>
-      <c r="H34" s="103"/>
-      <c r="I34" s="104"/>
+      <c r="B34" s="96"/>
+      <c r="C34" s="97"/>
+      <c r="D34" s="97"/>
+      <c r="E34" s="97"/>
+      <c r="F34" s="97"/>
+      <c r="G34" s="97"/>
+      <c r="H34" s="97"/>
+      <c r="I34" s="98"/>
       <c r="J34" s="70"/>
       <c r="K34" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L34" s="72"/>
-      <c r="M34" s="98"/>
-      <c r="N34" s="99"/>
+      <c r="M34" s="118"/>
+      <c r="N34" s="119"/>
     </row>
     <row r="35" spans="1:14" ht="13.5" customHeight="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="123"/>
-      <c r="C35" s="103"/>
-      <c r="D35" s="103"/>
-      <c r="E35" s="103"/>
-      <c r="F35" s="103"/>
-      <c r="G35" s="103"/>
-      <c r="H35" s="103"/>
-      <c r="I35" s="104"/>
+      <c r="B35" s="96"/>
+      <c r="C35" s="97"/>
+      <c r="D35" s="97"/>
+      <c r="E35" s="97"/>
+      <c r="F35" s="97"/>
+      <c r="G35" s="97"/>
+      <c r="H35" s="97"/>
+      <c r="I35" s="98"/>
       <c r="J35" s="70"/>
       <c r="K35" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L35" s="72"/>
-      <c r="M35" s="98"/>
-      <c r="N35" s="99"/>
+      <c r="M35" s="118"/>
+      <c r="N35" s="119"/>
     </row>
     <row r="36" spans="1:14" ht="13.5" customHeight="1">
       <c r="A36" s="69"/>
-      <c r="B36" s="123"/>
-      <c r="C36" s="103"/>
-      <c r="D36" s="103"/>
-      <c r="E36" s="103"/>
-      <c r="F36" s="103"/>
-      <c r="G36" s="103"/>
-      <c r="H36" s="103"/>
-      <c r="I36" s="104"/>
+      <c r="B36" s="96"/>
+      <c r="C36" s="97"/>
+      <c r="D36" s="97"/>
+      <c r="E36" s="97"/>
+      <c r="F36" s="97"/>
+      <c r="G36" s="97"/>
+      <c r="H36" s="97"/>
+      <c r="I36" s="98"/>
       <c r="J36" s="70"/>
       <c r="K36" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L36" s="72"/>
-      <c r="M36" s="98"/>
-      <c r="N36" s="99"/>
+      <c r="M36" s="118"/>
+      <c r="N36" s="119"/>
     </row>
     <row r="37" spans="1:14" ht="13.5" customHeight="1">
       <c r="A37" s="69"/>
-      <c r="B37" s="123"/>
-      <c r="C37" s="103"/>
-      <c r="D37" s="103"/>
-      <c r="E37" s="103"/>
-      <c r="F37" s="103"/>
-      <c r="G37" s="103"/>
-      <c r="H37" s="103"/>
-      <c r="I37" s="104"/>
+      <c r="B37" s="96"/>
+      <c r="C37" s="97"/>
+      <c r="D37" s="97"/>
+      <c r="E37" s="97"/>
+      <c r="F37" s="97"/>
+      <c r="G37" s="97"/>
+      <c r="H37" s="97"/>
+      <c r="I37" s="98"/>
       <c r="J37" s="70"/>
       <c r="K37" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L37" s="72"/>
-      <c r="M37" s="98"/>
-      <c r="N37" s="99"/>
+      <c r="M37" s="118"/>
+      <c r="N37" s="119"/>
     </row>
     <row r="38" spans="1:14" ht="13.5" customHeight="1">
       <c r="A38" s="69"/>
-      <c r="B38" s="123"/>
-      <c r="C38" s="103"/>
-      <c r="D38" s="103"/>
-      <c r="E38" s="103"/>
-      <c r="F38" s="103"/>
-      <c r="G38" s="103"/>
-      <c r="H38" s="103"/>
-      <c r="I38" s="104"/>
+      <c r="B38" s="96"/>
+      <c r="C38" s="97"/>
+      <c r="D38" s="97"/>
+      <c r="E38" s="97"/>
+      <c r="F38" s="97"/>
+      <c r="G38" s="97"/>
+      <c r="H38" s="97"/>
+      <c r="I38" s="98"/>
       <c r="J38" s="70"/>
       <c r="K38" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L38" s="72"/>
-      <c r="M38" s="98"/>
-      <c r="N38" s="99"/>
+      <c r="M38" s="118"/>
+      <c r="N38" s="119"/>
     </row>
     <row r="39" spans="1:14" ht="13.5" customHeight="1">
       <c r="A39" s="69"/>
-      <c r="B39" s="123"/>
-      <c r="C39" s="103"/>
-      <c r="D39" s="103"/>
-      <c r="E39" s="103"/>
-      <c r="F39" s="103"/>
-      <c r="G39" s="103"/>
-      <c r="H39" s="103"/>
-      <c r="I39" s="104"/>
+      <c r="B39" s="96"/>
+      <c r="C39" s="97"/>
+      <c r="D39" s="97"/>
+      <c r="E39" s="97"/>
+      <c r="F39" s="97"/>
+      <c r="G39" s="97"/>
+      <c r="H39" s="97"/>
+      <c r="I39" s="98"/>
       <c r="J39" s="70"/>
       <c r="K39" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L39" s="72"/>
-      <c r="M39" s="98"/>
-      <c r="N39" s="99"/>
+      <c r="M39" s="118"/>
+      <c r="N39" s="119"/>
     </row>
     <row r="40" spans="1:14" ht="13.5" customHeight="1">
       <c r="A40" s="69"/>
-      <c r="B40" s="123"/>
-      <c r="C40" s="103"/>
-      <c r="D40" s="103"/>
-      <c r="E40" s="103"/>
-      <c r="F40" s="103"/>
-      <c r="G40" s="103"/>
-      <c r="H40" s="103"/>
-      <c r="I40" s="104"/>
+      <c r="B40" s="96"/>
+      <c r="C40" s="97"/>
+      <c r="D40" s="97"/>
+      <c r="E40" s="97"/>
+      <c r="F40" s="97"/>
+      <c r="G40" s="97"/>
+      <c r="H40" s="97"/>
+      <c r="I40" s="98"/>
       <c r="J40" s="70"/>
       <c r="K40" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L40" s="72"/>
-      <c r="M40" s="98"/>
-      <c r="N40" s="99"/>
+      <c r="M40" s="118"/>
+      <c r="N40" s="119"/>
     </row>
     <row r="41" spans="1:14" ht="13.5" customHeight="1">
       <c r="A41" s="74"/>
-      <c r="B41" s="124"/>
-      <c r="C41" s="125"/>
-      <c r="D41" s="125"/>
-      <c r="E41" s="125"/>
-      <c r="F41" s="125"/>
-      <c r="G41" s="125"/>
-      <c r="H41" s="125"/>
-      <c r="I41" s="126"/>
+      <c r="B41" s="130"/>
+      <c r="C41" s="131"/>
+      <c r="D41" s="131"/>
+      <c r="E41" s="131"/>
+      <c r="F41" s="131"/>
+      <c r="G41" s="131"/>
+      <c r="H41" s="131"/>
+      <c r="I41" s="132"/>
       <c r="J41" s="75"/>
       <c r="K41" s="76">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L41" s="77"/>
-      <c r="M41" s="109"/>
-      <c r="N41" s="110"/>
+      <c r="M41" s="116"/>
+      <c r="N41" s="117"/>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
       <c r="A42" s="78"/>
@@ -4175,20 +4076,32 @@
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="M3:N4"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="B39:I39"/>
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="D23:I25"/>
+    <mergeCell ref="M37:N37"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="M40:N40"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="M34:N34"/>
     <mergeCell ref="M41:N41"/>
     <mergeCell ref="M35:N35"/>
     <mergeCell ref="D7:G7"/>
@@ -4205,32 +4118,20 @@
     <mergeCell ref="M30:N30"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B37:I37"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="M40:N40"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="D23:I25"/>
-    <mergeCell ref="M37:N37"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A14:I14"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="M3:N4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A9">

</xml_diff>

<commit_message>
Se cambio el QR de plantilla y TOD comm
</commit_message>
<xml_diff>
--- a/netlify/functions/plantilla.xlsx
+++ b/netlify/functions/plantilla.xlsx
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
   <si>
     <t>UNIDAD:</t>
   </si>
@@ -594,9 +594,6 @@
     </r>
   </si>
   <si>
-    <t>Pdte.(a) o Lider de Organización              Rendirá ctas. del gasto</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="8"/>
@@ -636,6 +633,81 @@
   </si>
   <si>
     <t xml:space="preserve">Nom:                                        </t>
+  </si>
+  <si>
+    <r>
+      <t>Aceptamos al FIRMAR el formulario:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Que una vez realizado la actividad, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>presentaremos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> hasta los siguientes </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>7 dias</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, las FACTURAS, comprobantes de pagos o compras. Y </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>dejar limpio</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>s los ambientes usados para dicha actividad, dejando la basura en los contenedores.</t>
+    </r>
+  </si>
+  <si>
+    <t>Pdte.(a) o Lider de Organización        Rendirá ctas. del gasto</t>
   </si>
 </sst>
 </file>
@@ -1624,7 +1696,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1839,29 +1911,72 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1877,93 +1992,56 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="20" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="45" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="45" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2004,19 +2082,19 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>178636</xdr:colOff>
+      <xdr:colOff>53855</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>8466</xdr:rowOff>
+      <xdr:rowOff>31420</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>250371</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>24378</xdr:rowOff>
+      <xdr:colOff>272701</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>15089</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2" descr="C:\Users\DELL 2021\Documents\IGLESIA\qr web sis presup.png"/>
+        <xdr:cNvPr id="5" name="Imagen 4" descr="C:\Users\DELL 2021\Documents\IGLESIA\QR directo a web sis presup.png"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -2036,8 +2114,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="178636" y="3998080"/>
-          <a:ext cx="643235" cy="658169"/>
+          <a:off x="53855" y="3973450"/>
+          <a:ext cx="792232" cy="790936"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2382,20 +2460,20 @@
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="107" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
+      <c r="C1" s="128" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
       <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="107"/>
-      <c r="I1" s="108"/>
+      <c r="H1" s="128"/>
+      <c r="I1" s="129"/>
       <c r="J1" s="4"/>
-      <c r="L1" s="109"/>
-      <c r="M1" s="100"/>
-      <c r="N1" s="100"/>
+      <c r="L1" s="130"/>
+      <c r="M1" s="113"/>
+      <c r="N1" s="113"/>
     </row>
     <row r="2" spans="1:14" ht="13.5" customHeight="1">
       <c r="A2" s="6"/>
@@ -2407,9 +2485,9 @@
         <v>3</v>
       </c>
       <c r="K2" s="8"/>
-      <c r="L2" s="110"/>
-      <c r="M2" s="111"/>
-      <c r="N2" s="111"/>
+      <c r="L2" s="131"/>
+      <c r="M2" s="132"/>
+      <c r="N2" s="132"/>
     </row>
     <row r="3" spans="1:14" ht="13.5" customHeight="1">
       <c r="A3" s="9" t="s">
@@ -2420,10 +2498,10 @@
         <v>5</v>
       </c>
       <c r="L3" s="10"/>
-      <c r="M3" s="112" t="s">
+      <c r="M3" s="133" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="113"/>
+      <c r="N3" s="134"/>
     </row>
     <row r="4" spans="1:14" ht="13.5" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -2438,12 +2516,12 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
       <c r="J4" s="11"/>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="154" t="s">
         <v>8</v>
       </c>
       <c r="L4" s="13"/>
-      <c r="M4" s="114"/>
-      <c r="N4" s="115"/>
+      <c r="M4" s="135"/>
+      <c r="N4" s="136"/>
     </row>
     <row r="5" spans="1:14" ht="13.5" customHeight="1">
       <c r="A5" s="9" t="s">
@@ -2452,11 +2530,11 @@
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="99"/>
-      <c r="F5" s="100"/>
-      <c r="G5" s="100"/>
-      <c r="H5" s="100"/>
-      <c r="I5" s="100"/>
+      <c r="E5" s="115"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="113"/>
+      <c r="I5" s="113"/>
       <c r="J5" s="4"/>
       <c r="K5" s="14" t="s">
         <v>10</v>
@@ -2472,15 +2550,15 @@
         <v>12</v>
       </c>
       <c r="B6" s="9"/>
-      <c r="C6" s="120"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="113"/>
+      <c r="E6" s="113"/>
+      <c r="F6" s="113"/>
       <c r="G6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="121"/>
-      <c r="I6" s="119"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="99"/>
       <c r="J6" s="4"/>
       <c r="K6" s="14" t="s">
         <v>14</v>
@@ -2497,10 +2575,10 @@
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="99"/>
-      <c r="E7" s="100"/>
-      <c r="F7" s="100"/>
-      <c r="G7" s="100"/>
+      <c r="D7" s="115"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="H7" s="9" t="s">
         <v>17</v>
       </c>
@@ -2509,8 +2587,8 @@
       <c r="K7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="122"/>
-      <c r="M7" s="123"/>
+      <c r="L7" s="116"/>
+      <c r="M7" s="117"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:14" ht="13.5" customHeight="1">
@@ -2519,7 +2597,7 @@
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G8" s="9"/>
       <c r="H8" s="9"/>
@@ -2528,19 +2606,19 @@
         <v>21</v>
       </c>
       <c r="K8" s="21"/>
-      <c r="L8" s="126"/>
-      <c r="M8" s="97"/>
-      <c r="N8" s="97"/>
+      <c r="L8" s="120"/>
+      <c r="M8" s="103"/>
+      <c r="N8" s="103"/>
     </row>
     <row r="9" spans="1:14" ht="13.5" customHeight="1">
       <c r="A9" s="94" t="s">
-        <v>73</v>
-      </c>
-      <c r="C9" s="99"/>
-      <c r="D9" s="100"/>
-      <c r="E9" s="100"/>
-      <c r="F9" s="100"/>
-      <c r="G9" s="100"/>
+        <v>72</v>
+      </c>
+      <c r="C9" s="115"/>
+      <c r="D9" s="113"/>
+      <c r="E9" s="113"/>
+      <c r="F9" s="113"/>
+      <c r="G9" s="113"/>
       <c r="J9" s="22" t="s">
         <v>68</v>
       </c>
@@ -2577,40 +2655,40 @@
       <c r="N11" s="28"/>
     </row>
     <row r="12" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A12" s="101"/>
-      <c r="B12" s="101"/>
-      <c r="C12" s="101"/>
-      <c r="D12" s="101"/>
-      <c r="E12" s="101"/>
-      <c r="F12" s="101"/>
-      <c r="G12" s="101"/>
-      <c r="H12" s="101"/>
-      <c r="I12" s="102"/>
+      <c r="A12" s="137"/>
+      <c r="B12" s="137"/>
+      <c r="C12" s="137"/>
+      <c r="D12" s="137"/>
+      <c r="E12" s="137"/>
+      <c r="F12" s="137"/>
+      <c r="G12" s="137"/>
+      <c r="H12" s="137"/>
+      <c r="I12" s="138"/>
       <c r="J12" s="27"/>
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A13" s="101"/>
-      <c r="B13" s="101"/>
-      <c r="C13" s="101"/>
-      <c r="D13" s="101"/>
-      <c r="E13" s="101"/>
-      <c r="F13" s="101"/>
-      <c r="G13" s="101"/>
-      <c r="H13" s="101"/>
-      <c r="I13" s="102"/>
+      <c r="A13" s="137"/>
+      <c r="B13" s="137"/>
+      <c r="C13" s="137"/>
+      <c r="D13" s="137"/>
+      <c r="E13" s="137"/>
+      <c r="F13" s="137"/>
+      <c r="G13" s="137"/>
+      <c r="H13" s="137"/>
+      <c r="I13" s="138"/>
       <c r="J13" s="11"/>
     </row>
     <row r="14" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A14" s="101"/>
-      <c r="B14" s="101"/>
-      <c r="C14" s="101"/>
-      <c r="D14" s="101"/>
-      <c r="E14" s="101"/>
-      <c r="F14" s="101"/>
-      <c r="G14" s="101"/>
-      <c r="H14" s="101"/>
-      <c r="I14" s="102"/>
+      <c r="A14" s="137"/>
+      <c r="B14" s="137"/>
+      <c r="C14" s="137"/>
+      <c r="D14" s="137"/>
+      <c r="E14" s="137"/>
+      <c r="F14" s="137"/>
+      <c r="G14" s="137"/>
+      <c r="H14" s="137"/>
+      <c r="I14" s="138"/>
       <c r="J14" s="29"/>
       <c r="K14" s="6"/>
       <c r="L14" s="30"/>
@@ -2618,33 +2696,33 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A15" s="101"/>
-      <c r="B15" s="101"/>
-      <c r="C15" s="101"/>
-      <c r="D15" s="101"/>
-      <c r="E15" s="101"/>
-      <c r="F15" s="101"/>
-      <c r="G15" s="101"/>
-      <c r="H15" s="101"/>
-      <c r="I15" s="102"/>
+      <c r="A15" s="137"/>
+      <c r="B15" s="137"/>
+      <c r="C15" s="137"/>
+      <c r="D15" s="137"/>
+      <c r="E15" s="137"/>
+      <c r="F15" s="137"/>
+      <c r="G15" s="137"/>
+      <c r="H15" s="137"/>
+      <c r="I15" s="138"/>
       <c r="J15" s="29" t="s">
         <v>27</v>
       </c>
       <c r="L15" s="32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N15" s="28"/>
     </row>
     <row r="16" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A16" s="101"/>
-      <c r="B16" s="101"/>
-      <c r="C16" s="101"/>
-      <c r="D16" s="101"/>
-      <c r="E16" s="101"/>
-      <c r="F16" s="101"/>
-      <c r="G16" s="101"/>
-      <c r="H16" s="101"/>
-      <c r="I16" s="102"/>
+      <c r="A16" s="137"/>
+      <c r="B16" s="137"/>
+      <c r="C16" s="137"/>
+      <c r="D16" s="137"/>
+      <c r="E16" s="137"/>
+      <c r="F16" s="137"/>
+      <c r="G16" s="137"/>
+      <c r="H16" s="137"/>
+      <c r="I16" s="138"/>
       <c r="J16" s="33" t="s">
         <v>28</v>
       </c>
@@ -2652,21 +2730,21 @@
         <v>66</v>
       </c>
       <c r="L16" s="35"/>
-      <c r="M16" s="150" t="s">
+      <c r="M16" s="100" t="s">
         <v>67</v>
       </c>
-      <c r="N16" s="151"/>
+      <c r="N16" s="101"/>
     </row>
     <row r="17" spans="1:14" ht="14.4">
-      <c r="A17" s="101"/>
-      <c r="B17" s="101"/>
-      <c r="C17" s="101"/>
-      <c r="D17" s="101"/>
-      <c r="E17" s="101"/>
-      <c r="F17" s="101"/>
-      <c r="G17" s="101"/>
-      <c r="H17" s="101"/>
-      <c r="I17" s="102"/>
+      <c r="A17" s="137"/>
+      <c r="B17" s="137"/>
+      <c r="C17" s="137"/>
+      <c r="D17" s="137"/>
+      <c r="E17" s="137"/>
+      <c r="F17" s="137"/>
+      <c r="G17" s="137"/>
+      <c r="H17" s="137"/>
+      <c r="I17" s="138"/>
       <c r="J17" s="36" t="s">
         <v>29</v>
       </c>
@@ -2676,28 +2754,28 @@
         <v>30</v>
       </c>
       <c r="J18" s="38"/>
-      <c r="K18" s="124" t="s">
+      <c r="K18" s="102" t="s">
         <v>31</v>
       </c>
-      <c r="L18" s="97"/>
-      <c r="M18" s="97"/>
-      <c r="N18" s="98"/>
+      <c r="L18" s="103"/>
+      <c r="M18" s="103"/>
+      <c r="N18" s="104"/>
     </row>
     <row r="19" spans="1:14" ht="13.5" customHeight="1">
       <c r="J19" s="38"/>
-      <c r="K19" s="124" t="s">
+      <c r="K19" s="102" t="s">
         <v>32</v>
       </c>
-      <c r="L19" s="97"/>
-      <c r="M19" s="97"/>
-      <c r="N19" s="98"/>
+      <c r="L19" s="103"/>
+      <c r="M19" s="103"/>
+      <c r="N19" s="104"/>
     </row>
     <row r="20" spans="1:14" ht="13.5" customHeight="1">
-      <c r="B20" s="125"/>
-      <c r="C20" s="104"/>
-      <c r="D20" s="104"/>
-      <c r="E20" s="104"/>
-      <c r="F20" s="104"/>
+      <c r="B20" s="118"/>
+      <c r="C20" s="119"/>
+      <c r="D20" s="119"/>
+      <c r="E20" s="119"/>
+      <c r="F20" s="119"/>
       <c r="H20" s="39"/>
       <c r="J20" s="40"/>
       <c r="K20" s="41"/>
@@ -2707,64 +2785,63 @@
     </row>
     <row r="21" spans="1:14" ht="20.25" customHeight="1">
       <c r="B21" s="32" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D21" s="43"/>
       <c r="E21" s="26"/>
       <c r="J21" s="38"/>
-      <c r="K21" s="124" t="s">
+      <c r="K21" s="102" t="s">
         <v>34</v>
       </c>
-      <c r="L21" s="97"/>
-      <c r="M21" s="97"/>
-      <c r="N21" s="98"/>
+      <c r="L21" s="103"/>
+      <c r="M21" s="103"/>
+      <c r="N21" s="104"/>
     </row>
     <row r="22" spans="1:14" ht="23.25" customHeight="1">
       <c r="B22" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="142"/>
+      <c r="D22" s="142"/>
+      <c r="E22" s="142"/>
+      <c r="G22" s="139"/>
+      <c r="H22" s="140"/>
+      <c r="J22" s="38"/>
+      <c r="K22" s="102" t="s">
+        <v>36</v>
+      </c>
+      <c r="L22" s="103"/>
+      <c r="M22" s="103"/>
+      <c r="N22" s="104"/>
+    </row>
+    <row r="23" spans="1:14" ht="17.25" customHeight="1">
+      <c r="C23" s="44"/>
+      <c r="D23" s="155" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="106"/>
-      <c r="D22" s="106"/>
-      <c r="E22" s="106"/>
-      <c r="G22" s="152"/>
-      <c r="H22" s="153"/>
-      <c r="J22" s="38"/>
-      <c r="K22" s="124" t="s">
-        <v>36</v>
-      </c>
-      <c r="L22" s="97"/>
-      <c r="M22" s="97"/>
-      <c r="N22" s="98"/>
-    </row>
-    <row r="23" spans="1:14" ht="17.25" customHeight="1">
-      <c r="B23" s="44"/>
-      <c r="C23" s="44"/>
-      <c r="D23" s="105" t="s">
-        <v>37</v>
-      </c>
-      <c r="E23" s="104"/>
-      <c r="F23" s="104"/>
-      <c r="G23" s="104"/>
-      <c r="H23" s="104"/>
-      <c r="I23" s="104"/>
+      <c r="E23" s="155"/>
+      <c r="F23" s="155"/>
+      <c r="G23" s="155"/>
+      <c r="H23" s="155"/>
+      <c r="I23" s="155"/>
       <c r="J23" s="38"/>
-      <c r="K23" s="137" t="s">
+      <c r="K23" s="105" t="s">
         <v>38</v>
       </c>
-      <c r="L23" s="97"/>
-      <c r="M23" s="97"/>
-      <c r="N23" s="98"/>
+      <c r="L23" s="103"/>
+      <c r="M23" s="103"/>
+      <c r="N23" s="104"/>
     </row>
     <row r="24" spans="1:14" ht="13.5" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="44"/>
       <c r="C24" s="44"/>
-      <c r="D24" s="104"/>
-      <c r="E24" s="104"/>
-      <c r="F24" s="104"/>
-      <c r="G24" s="104"/>
-      <c r="H24" s="104"/>
-      <c r="I24" s="104"/>
+      <c r="D24" s="155"/>
+      <c r="E24" s="155"/>
+      <c r="F24" s="155"/>
+      <c r="G24" s="155"/>
+      <c r="H24" s="155"/>
+      <c r="I24" s="155"/>
       <c r="J24" s="40"/>
       <c r="K24" s="41"/>
       <c r="L24" s="42"/>
@@ -2775,19 +2852,25 @@
       <c r="A25" s="44"/>
       <c r="B25" s="44"/>
       <c r="C25" s="44"/>
-      <c r="D25" s="104"/>
-      <c r="E25" s="104"/>
-      <c r="F25" s="104"/>
-      <c r="G25" s="104"/>
-      <c r="H25" s="104"/>
-      <c r="I25" s="104"/>
+      <c r="D25" s="155"/>
+      <c r="E25" s="155"/>
+      <c r="F25" s="155"/>
+      <c r="G25" s="155"/>
+      <c r="H25" s="155"/>
+      <c r="I25" s="155"/>
       <c r="J25" s="38"/>
-      <c r="K25" s="137"/>
-      <c r="L25" s="138"/>
-      <c r="M25" s="138"/>
-      <c r="N25" s="139"/>
+      <c r="K25" s="105"/>
+      <c r="L25" s="106"/>
+      <c r="M25" s="106"/>
+      <c r="N25" s="107"/>
     </row>
     <row r="26" spans="1:14" ht="13.5" customHeight="1">
+      <c r="D26" s="155"/>
+      <c r="E26" s="155"/>
+      <c r="F26" s="155"/>
+      <c r="G26" s="155"/>
+      <c r="H26" s="155"/>
+      <c r="I26" s="155"/>
       <c r="J26" s="38"/>
       <c r="K26" s="45"/>
       <c r="L26" s="46"/>
@@ -2834,218 +2917,218 @@
       <c r="L28" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="M28" s="140" t="s">
+      <c r="M28" s="108" t="s">
         <v>46</v>
       </c>
-      <c r="N28" s="141"/>
+      <c r="N28" s="109"/>
     </row>
     <row r="29" spans="1:14" ht="13.5" customHeight="1">
       <c r="A29" s="65"/>
-      <c r="B29" s="127"/>
-      <c r="C29" s="128"/>
-      <c r="D29" s="128"/>
-      <c r="E29" s="128"/>
-      <c r="F29" s="128"/>
-      <c r="G29" s="128"/>
-      <c r="H29" s="128"/>
-      <c r="I29" s="129"/>
+      <c r="B29" s="121"/>
+      <c r="C29" s="122"/>
+      <c r="D29" s="122"/>
+      <c r="E29" s="122"/>
+      <c r="F29" s="122"/>
+      <c r="G29" s="122"/>
+      <c r="H29" s="122"/>
+      <c r="I29" s="123"/>
       <c r="J29" s="66"/>
       <c r="K29" s="67"/>
       <c r="L29" s="68"/>
-      <c r="M29" s="133"/>
-      <c r="N29" s="134"/>
+      <c r="M29" s="96"/>
+      <c r="N29" s="97"/>
     </row>
     <row r="30" spans="1:14" ht="13.5" customHeight="1">
       <c r="A30" s="69"/>
-      <c r="B30" s="96"/>
-      <c r="C30" s="97"/>
-      <c r="D30" s="97"/>
-      <c r="E30" s="97"/>
-      <c r="F30" s="97"/>
-      <c r="G30" s="97"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="98"/>
+      <c r="B30" s="124"/>
+      <c r="C30" s="103"/>
+      <c r="D30" s="103"/>
+      <c r="E30" s="103"/>
+      <c r="F30" s="103"/>
+      <c r="G30" s="103"/>
+      <c r="H30" s="103"/>
+      <c r="I30" s="104"/>
       <c r="J30" s="70"/>
       <c r="K30" s="71"/>
       <c r="L30" s="72"/>
-      <c r="M30" s="118"/>
-      <c r="N30" s="119"/>
+      <c r="M30" s="98"/>
+      <c r="N30" s="99"/>
     </row>
     <row r="31" spans="1:14" ht="13.5" customHeight="1">
       <c r="A31" s="69"/>
-      <c r="B31" s="96"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="97"/>
-      <c r="E31" s="97"/>
-      <c r="F31" s="97"/>
-      <c r="G31" s="97"/>
-      <c r="H31" s="97"/>
-      <c r="I31" s="98"/>
+      <c r="B31" s="124"/>
+      <c r="C31" s="103"/>
+      <c r="D31" s="103"/>
+      <c r="E31" s="103"/>
+      <c r="F31" s="103"/>
+      <c r="G31" s="103"/>
+      <c r="H31" s="103"/>
+      <c r="I31" s="104"/>
       <c r="J31" s="73"/>
       <c r="K31" s="71"/>
       <c r="L31" s="72"/>
-      <c r="M31" s="118"/>
-      <c r="N31" s="119"/>
+      <c r="M31" s="98"/>
+      <c r="N31" s="99"/>
     </row>
     <row r="32" spans="1:14" ht="13.5" customHeight="1">
       <c r="A32" s="69"/>
-      <c r="B32" s="96"/>
-      <c r="C32" s="97"/>
-      <c r="D32" s="97"/>
-      <c r="E32" s="97"/>
-      <c r="F32" s="97"/>
-      <c r="G32" s="97"/>
-      <c r="H32" s="97"/>
-      <c r="I32" s="98"/>
+      <c r="B32" s="124"/>
+      <c r="C32" s="103"/>
+      <c r="D32" s="103"/>
+      <c r="E32" s="103"/>
+      <c r="F32" s="103"/>
+      <c r="G32" s="103"/>
+      <c r="H32" s="103"/>
+      <c r="I32" s="104"/>
       <c r="J32" s="73"/>
       <c r="K32" s="71"/>
       <c r="L32" s="72"/>
-      <c r="M32" s="118"/>
-      <c r="N32" s="119"/>
+      <c r="M32" s="98"/>
+      <c r="N32" s="99"/>
     </row>
     <row r="33" spans="1:14" ht="13.5" customHeight="1">
       <c r="A33" s="69"/>
-      <c r="B33" s="96"/>
-      <c r="C33" s="97"/>
-      <c r="D33" s="97"/>
-      <c r="E33" s="97"/>
-      <c r="F33" s="97"/>
-      <c r="G33" s="97"/>
-      <c r="H33" s="97"/>
-      <c r="I33" s="98"/>
+      <c r="B33" s="124"/>
+      <c r="C33" s="103"/>
+      <c r="D33" s="103"/>
+      <c r="E33" s="103"/>
+      <c r="F33" s="103"/>
+      <c r="G33" s="103"/>
+      <c r="H33" s="103"/>
+      <c r="I33" s="104"/>
       <c r="J33" s="73"/>
       <c r="K33" s="71"/>
       <c r="L33" s="72"/>
-      <c r="M33" s="118"/>
-      <c r="N33" s="119"/>
+      <c r="M33" s="98"/>
+      <c r="N33" s="99"/>
     </row>
     <row r="34" spans="1:14" ht="13.5" customHeight="1">
       <c r="A34" s="69"/>
-      <c r="B34" s="96"/>
-      <c r="C34" s="97"/>
-      <c r="D34" s="97"/>
-      <c r="E34" s="97"/>
-      <c r="F34" s="97"/>
-      <c r="G34" s="97"/>
-      <c r="H34" s="97"/>
-      <c r="I34" s="98"/>
+      <c r="B34" s="124"/>
+      <c r="C34" s="103"/>
+      <c r="D34" s="103"/>
+      <c r="E34" s="103"/>
+      <c r="F34" s="103"/>
+      <c r="G34" s="103"/>
+      <c r="H34" s="103"/>
+      <c r="I34" s="104"/>
       <c r="J34" s="70"/>
       <c r="K34" s="71"/>
       <c r="L34" s="72"/>
-      <c r="M34" s="118"/>
-      <c r="N34" s="119"/>
+      <c r="M34" s="98"/>
+      <c r="N34" s="99"/>
     </row>
     <row r="35" spans="1:14" ht="13.5" customHeight="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="96"/>
-      <c r="C35" s="97"/>
-      <c r="D35" s="97"/>
-      <c r="E35" s="97"/>
-      <c r="F35" s="97"/>
-      <c r="G35" s="97"/>
-      <c r="H35" s="97"/>
-      <c r="I35" s="98"/>
+      <c r="B35" s="124"/>
+      <c r="C35" s="103"/>
+      <c r="D35" s="103"/>
+      <c r="E35" s="103"/>
+      <c r="F35" s="103"/>
+      <c r="G35" s="103"/>
+      <c r="H35" s="103"/>
+      <c r="I35" s="104"/>
       <c r="J35" s="70"/>
       <c r="K35" s="71"/>
       <c r="L35" s="72"/>
-      <c r="M35" s="118"/>
-      <c r="N35" s="119"/>
+      <c r="M35" s="98"/>
+      <c r="N35" s="99"/>
     </row>
     <row r="36" spans="1:14" ht="13.5" customHeight="1">
       <c r="A36" s="69"/>
-      <c r="B36" s="96"/>
-      <c r="C36" s="97"/>
-      <c r="D36" s="97"/>
-      <c r="E36" s="97"/>
-      <c r="F36" s="97"/>
-      <c r="G36" s="97"/>
-      <c r="H36" s="97"/>
-      <c r="I36" s="98"/>
+      <c r="B36" s="124"/>
+      <c r="C36" s="103"/>
+      <c r="D36" s="103"/>
+      <c r="E36" s="103"/>
+      <c r="F36" s="103"/>
+      <c r="G36" s="103"/>
+      <c r="H36" s="103"/>
+      <c r="I36" s="104"/>
       <c r="J36" s="70"/>
       <c r="K36" s="71"/>
       <c r="L36" s="72"/>
-      <c r="M36" s="118"/>
-      <c r="N36" s="119"/>
+      <c r="M36" s="98"/>
+      <c r="N36" s="99"/>
     </row>
     <row r="37" spans="1:14" ht="13.5" customHeight="1">
       <c r="A37" s="69"/>
-      <c r="B37" s="96"/>
-      <c r="C37" s="97"/>
-      <c r="D37" s="97"/>
-      <c r="E37" s="97"/>
-      <c r="F37" s="97"/>
-      <c r="G37" s="97"/>
-      <c r="H37" s="97"/>
-      <c r="I37" s="98"/>
+      <c r="B37" s="124"/>
+      <c r="C37" s="103"/>
+      <c r="D37" s="103"/>
+      <c r="E37" s="103"/>
+      <c r="F37" s="103"/>
+      <c r="G37" s="103"/>
+      <c r="H37" s="103"/>
+      <c r="I37" s="104"/>
       <c r="J37" s="70"/>
       <c r="K37" s="71"/>
       <c r="L37" s="72"/>
-      <c r="M37" s="118"/>
-      <c r="N37" s="119"/>
+      <c r="M37" s="98"/>
+      <c r="N37" s="99"/>
     </row>
     <row r="38" spans="1:14" ht="13.5" customHeight="1">
       <c r="A38" s="69"/>
-      <c r="B38" s="96"/>
-      <c r="C38" s="97"/>
-      <c r="D38" s="97"/>
-      <c r="E38" s="97"/>
-      <c r="F38" s="97"/>
-      <c r="G38" s="97"/>
-      <c r="H38" s="97"/>
-      <c r="I38" s="98"/>
+      <c r="B38" s="124"/>
+      <c r="C38" s="103"/>
+      <c r="D38" s="103"/>
+      <c r="E38" s="103"/>
+      <c r="F38" s="103"/>
+      <c r="G38" s="103"/>
+      <c r="H38" s="103"/>
+      <c r="I38" s="104"/>
       <c r="J38" s="70"/>
       <c r="K38" s="71"/>
       <c r="L38" s="72"/>
-      <c r="M38" s="118"/>
-      <c r="N38" s="119"/>
+      <c r="M38" s="98"/>
+      <c r="N38" s="99"/>
     </row>
     <row r="39" spans="1:14" ht="13.5" customHeight="1">
       <c r="A39" s="69"/>
-      <c r="B39" s="96"/>
-      <c r="C39" s="97"/>
-      <c r="D39" s="97"/>
-      <c r="E39" s="97"/>
-      <c r="F39" s="97"/>
-      <c r="G39" s="97"/>
-      <c r="H39" s="97"/>
-      <c r="I39" s="98"/>
+      <c r="B39" s="124"/>
+      <c r="C39" s="103"/>
+      <c r="D39" s="103"/>
+      <c r="E39" s="103"/>
+      <c r="F39" s="103"/>
+      <c r="G39" s="103"/>
+      <c r="H39" s="103"/>
+      <c r="I39" s="104"/>
       <c r="J39" s="70"/>
       <c r="K39" s="71"/>
       <c r="L39" s="72"/>
-      <c r="M39" s="118"/>
-      <c r="N39" s="119"/>
+      <c r="M39" s="98"/>
+      <c r="N39" s="99"/>
     </row>
     <row r="40" spans="1:14" ht="13.5" customHeight="1">
       <c r="A40" s="69"/>
-      <c r="B40" s="96"/>
-      <c r="C40" s="97"/>
-      <c r="D40" s="97"/>
-      <c r="E40" s="97"/>
-      <c r="F40" s="97"/>
-      <c r="G40" s="97"/>
-      <c r="H40" s="97"/>
-      <c r="I40" s="98"/>
+      <c r="B40" s="124"/>
+      <c r="C40" s="103"/>
+      <c r="D40" s="103"/>
+      <c r="E40" s="103"/>
+      <c r="F40" s="103"/>
+      <c r="G40" s="103"/>
+      <c r="H40" s="103"/>
+      <c r="I40" s="104"/>
       <c r="J40" s="70"/>
       <c r="K40" s="71"/>
       <c r="L40" s="72"/>
-      <c r="M40" s="118"/>
-      <c r="N40" s="119"/>
+      <c r="M40" s="98"/>
+      <c r="N40" s="99"/>
     </row>
     <row r="41" spans="1:14" ht="13.5" customHeight="1">
       <c r="A41" s="74"/>
-      <c r="B41" s="130"/>
-      <c r="C41" s="131"/>
-      <c r="D41" s="131"/>
-      <c r="E41" s="131"/>
-      <c r="F41" s="131"/>
-      <c r="G41" s="131"/>
-      <c r="H41" s="131"/>
-      <c r="I41" s="132"/>
+      <c r="B41" s="125"/>
+      <c r="C41" s="126"/>
+      <c r="D41" s="126"/>
+      <c r="E41" s="126"/>
+      <c r="F41" s="126"/>
+      <c r="G41" s="126"/>
+      <c r="H41" s="126"/>
+      <c r="I41" s="127"/>
       <c r="J41" s="75"/>
       <c r="K41" s="76"/>
       <c r="L41" s="77"/>
-      <c r="M41" s="116"/>
-      <c r="N41" s="117"/>
+      <c r="M41" s="110"/>
+      <c r="N41" s="111"/>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
       <c r="A42" s="78"/>
@@ -3145,23 +3228,24 @@
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="K18:N18"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="K22:N22"/>
-    <mergeCell ref="K23:N23"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="M37:N37"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A12:I17"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="D23:I26"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="M3:N4"/>
     <mergeCell ref="M41:N41"/>
     <mergeCell ref="M40:N40"/>
     <mergeCell ref="C6:F6"/>
@@ -3178,24 +3262,23 @@
     <mergeCell ref="B38:I38"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B41:I41"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="M3:N4"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A12:I17"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="D23:I25"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="M37:N37"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="K18:N18"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="K22:N22"/>
+    <mergeCell ref="K23:N23"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="M28:N28"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:E1 H1:I1 L2:N2 E5:I5 C6:F6 H6:I6 D7:G7 B8 L8 A12:I17 K16 M16:N16 B20:F20 C22 G22:H22">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
@@ -3241,21 +3324,21 @@
         <v>54</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
+      <c r="C1" s="128"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
       <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="107"/>
-      <c r="I1" s="108"/>
+      <c r="H1" s="128"/>
+      <c r="I1" s="129"/>
       <c r="J1" s="4"/>
       <c r="K1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="109"/>
-      <c r="M1" s="100"/>
-      <c r="N1" s="100"/>
+      <c r="L1" s="130"/>
+      <c r="M1" s="113"/>
+      <c r="N1" s="113"/>
     </row>
     <row r="2" spans="1:14" ht="13.5" customHeight="1">
       <c r="A2" s="6"/>
@@ -3267,9 +3350,9 @@
         <v>3</v>
       </c>
       <c r="K2" s="8"/>
-      <c r="L2" s="142"/>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
+      <c r="L2" s="153"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
     </row>
     <row r="3" spans="1:14" ht="13.5" customHeight="1">
       <c r="A3" s="9" t="s">
@@ -3280,10 +3363,10 @@
         <v>5</v>
       </c>
       <c r="L3" s="10"/>
-      <c r="M3" s="112" t="s">
+      <c r="M3" s="133" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="113"/>
+      <c r="N3" s="134"/>
     </row>
     <row r="4" spans="1:14" ht="13.5" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -3302,8 +3385,8 @@
         <v>8</v>
       </c>
       <c r="L4" s="13"/>
-      <c r="M4" s="114"/>
-      <c r="N4" s="115"/>
+      <c r="M4" s="135"/>
+      <c r="N4" s="136"/>
     </row>
     <row r="5" spans="1:14" ht="13.5" customHeight="1">
       <c r="A5" s="9" t="s">
@@ -3312,11 +3395,11 @@
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="99"/>
-      <c r="F5" s="100"/>
-      <c r="G5" s="100"/>
-      <c r="H5" s="100"/>
-      <c r="I5" s="100"/>
+      <c r="E5" s="115"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="113"/>
+      <c r="I5" s="113"/>
       <c r="J5" s="4"/>
       <c r="K5" s="14" t="s">
         <v>10</v>
@@ -3332,15 +3415,15 @@
         <v>12</v>
       </c>
       <c r="B6" s="9"/>
-      <c r="C6" s="120"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="113"/>
+      <c r="E6" s="113"/>
+      <c r="F6" s="113"/>
       <c r="G6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="121"/>
-      <c r="I6" s="119"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="99"/>
       <c r="J6" s="4"/>
       <c r="K6" s="14" t="s">
         <v>14</v>
@@ -3357,10 +3440,10 @@
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="99"/>
-      <c r="E7" s="100"/>
-      <c r="F7" s="100"/>
-      <c r="G7" s="100"/>
+      <c r="D7" s="115"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="H7" s="9" t="s">
         <v>17</v>
       </c>
@@ -3369,11 +3452,11 @@
       <c r="K7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="143">
+      <c r="L7" s="149">
         <f>SUM(L4:L6)+N5+N6</f>
         <v>0</v>
       </c>
-      <c r="M7" s="123"/>
+      <c r="M7" s="117"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:14" ht="13.5" customHeight="1">
@@ -3391,22 +3474,22 @@
         <v>21</v>
       </c>
       <c r="K8" s="21"/>
-      <c r="L8" s="126"/>
-      <c r="M8" s="97"/>
-      <c r="N8" s="97"/>
+      <c r="L8" s="120"/>
+      <c r="M8" s="103"/>
+      <c r="N8" s="103"/>
     </row>
     <row r="9" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A9" s="148" t="s">
+      <c r="A9" s="146" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="104"/>
-      <c r="C9" s="104"/>
-      <c r="D9" s="104"/>
-      <c r="E9" s="104"/>
-      <c r="F9" s="104"/>
-      <c r="G9" s="104"/>
-      <c r="H9" s="104"/>
-      <c r="I9" s="149"/>
+      <c r="B9" s="119"/>
+      <c r="C9" s="119"/>
+      <c r="D9" s="119"/>
+      <c r="E9" s="119"/>
+      <c r="F9" s="119"/>
+      <c r="G9" s="119"/>
+      <c r="H9" s="119"/>
+      <c r="I9" s="147"/>
       <c r="J9" s="22" t="s">
         <v>23</v>
       </c>
@@ -3441,40 +3524,40 @@
       <c r="N11" s="28"/>
     </row>
     <row r="12" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A12" s="145"/>
-      <c r="B12" s="100"/>
-      <c r="C12" s="100"/>
-      <c r="D12" s="100"/>
-      <c r="E12" s="100"/>
-      <c r="F12" s="100"/>
-      <c r="G12" s="100"/>
-      <c r="H12" s="100"/>
-      <c r="I12" s="108"/>
+      <c r="A12" s="143"/>
+      <c r="B12" s="113"/>
+      <c r="C12" s="113"/>
+      <c r="D12" s="113"/>
+      <c r="E12" s="113"/>
+      <c r="F12" s="113"/>
+      <c r="G12" s="113"/>
+      <c r="H12" s="113"/>
+      <c r="I12" s="129"/>
       <c r="J12" s="27"/>
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A13" s="146"/>
-      <c r="B13" s="97"/>
-      <c r="C13" s="97"/>
-      <c r="D13" s="97"/>
-      <c r="E13" s="97"/>
-      <c r="F13" s="97"/>
-      <c r="G13" s="97"/>
-      <c r="H13" s="97"/>
-      <c r="I13" s="119"/>
+      <c r="A13" s="144"/>
+      <c r="B13" s="103"/>
+      <c r="C13" s="103"/>
+      <c r="D13" s="103"/>
+      <c r="E13" s="103"/>
+      <c r="F13" s="103"/>
+      <c r="G13" s="103"/>
+      <c r="H13" s="103"/>
+      <c r="I13" s="99"/>
       <c r="J13" s="11"/>
     </row>
     <row r="14" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A14" s="146"/>
-      <c r="B14" s="97"/>
-      <c r="C14" s="97"/>
-      <c r="D14" s="97"/>
-      <c r="E14" s="97"/>
-      <c r="F14" s="97"/>
-      <c r="G14" s="97"/>
-      <c r="H14" s="97"/>
-      <c r="I14" s="119"/>
+      <c r="A14" s="144"/>
+      <c r="B14" s="103"/>
+      <c r="C14" s="103"/>
+      <c r="D14" s="103"/>
+      <c r="E14" s="103"/>
+      <c r="F14" s="103"/>
+      <c r="G14" s="103"/>
+      <c r="H14" s="103"/>
+      <c r="I14" s="99"/>
       <c r="J14" s="29"/>
       <c r="K14" s="6"/>
       <c r="L14" s="30"/>
@@ -3482,15 +3565,15 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A15" s="146"/>
-      <c r="B15" s="97"/>
-      <c r="C15" s="97"/>
-      <c r="D15" s="97"/>
-      <c r="E15" s="97"/>
-      <c r="F15" s="97"/>
-      <c r="G15" s="97"/>
-      <c r="H15" s="97"/>
-      <c r="I15" s="119"/>
+      <c r="A15" s="144"/>
+      <c r="B15" s="103"/>
+      <c r="C15" s="103"/>
+      <c r="D15" s="103"/>
+      <c r="E15" s="103"/>
+      <c r="F15" s="103"/>
+      <c r="G15" s="103"/>
+      <c r="H15" s="103"/>
+      <c r="I15" s="99"/>
       <c r="J15" s="29" t="s">
         <v>55</v>
       </c>
@@ -3501,33 +3584,33 @@
       <c r="N15" s="28"/>
     </row>
     <row r="16" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A16" s="146"/>
-      <c r="B16" s="97"/>
-      <c r="C16" s="97"/>
-      <c r="D16" s="97"/>
-      <c r="E16" s="97"/>
-      <c r="F16" s="97"/>
-      <c r="G16" s="97"/>
-      <c r="H16" s="97"/>
-      <c r="I16" s="119"/>
+      <c r="A16" s="144"/>
+      <c r="B16" s="103"/>
+      <c r="C16" s="103"/>
+      <c r="D16" s="103"/>
+      <c r="E16" s="103"/>
+      <c r="F16" s="103"/>
+      <c r="G16" s="103"/>
+      <c r="H16" s="103"/>
+      <c r="I16" s="99"/>
       <c r="J16" s="33" t="s">
         <v>28</v>
       </c>
       <c r="K16" s="34"/>
       <c r="L16" s="35"/>
-      <c r="M16" s="135"/>
-      <c r="N16" s="136"/>
+      <c r="M16" s="151"/>
+      <c r="N16" s="152"/>
     </row>
     <row r="17" spans="1:14" ht="14.4">
-      <c r="A17" s="147"/>
-      <c r="B17" s="104"/>
-      <c r="C17" s="104"/>
-      <c r="D17" s="104"/>
-      <c r="E17" s="104"/>
-      <c r="F17" s="104"/>
-      <c r="G17" s="104"/>
-      <c r="H17" s="104"/>
-      <c r="I17" s="104"/>
+      <c r="A17" s="145"/>
+      <c r="B17" s="119"/>
+      <c r="C17" s="119"/>
+      <c r="D17" s="119"/>
+      <c r="E17" s="119"/>
+      <c r="F17" s="119"/>
+      <c r="G17" s="119"/>
+      <c r="H17" s="119"/>
+      <c r="I17" s="119"/>
       <c r="J17" s="36" t="s">
         <v>29</v>
       </c>
@@ -3537,28 +3620,28 @@
         <v>30</v>
       </c>
       <c r="J18" s="38"/>
-      <c r="K18" s="144" t="s">
+      <c r="K18" s="150" t="s">
         <v>57</v>
       </c>
-      <c r="L18" s="97"/>
-      <c r="M18" s="97"/>
-      <c r="N18" s="98"/>
+      <c r="L18" s="103"/>
+      <c r="M18" s="103"/>
+      <c r="N18" s="104"/>
     </row>
     <row r="19" spans="1:14" ht="13.5" customHeight="1">
       <c r="J19" s="38"/>
-      <c r="K19" s="144" t="s">
+      <c r="K19" s="150" t="s">
         <v>58</v>
       </c>
-      <c r="L19" s="97"/>
-      <c r="M19" s="97"/>
-      <c r="N19" s="98"/>
+      <c r="L19" s="103"/>
+      <c r="M19" s="103"/>
+      <c r="N19" s="104"/>
     </row>
     <row r="20" spans="1:14" ht="13.5" customHeight="1">
-      <c r="B20" s="125"/>
-      <c r="C20" s="104"/>
-      <c r="D20" s="104"/>
-      <c r="E20" s="104"/>
-      <c r="F20" s="104"/>
+      <c r="B20" s="118"/>
+      <c r="C20" s="119"/>
+      <c r="D20" s="119"/>
+      <c r="E20" s="119"/>
+      <c r="F20" s="119"/>
       <c r="H20" s="39"/>
       <c r="J20" s="40"/>
       <c r="K20" s="41" t="s">
@@ -3575,59 +3658,59 @@
       <c r="D21" s="43"/>
       <c r="E21" s="26"/>
       <c r="J21" s="38"/>
-      <c r="K21" s="144" t="s">
+      <c r="K21" s="150" t="s">
         <v>60</v>
       </c>
-      <c r="L21" s="97"/>
-      <c r="M21" s="97"/>
-      <c r="N21" s="98"/>
+      <c r="L21" s="103"/>
+      <c r="M21" s="103"/>
+      <c r="N21" s="104"/>
     </row>
     <row r="22" spans="1:14" ht="17.25" customHeight="1">
       <c r="C22" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D22" s="106"/>
-      <c r="E22" s="104"/>
+      <c r="D22" s="142"/>
+      <c r="E22" s="119"/>
       <c r="F22" s="26"/>
-      <c r="G22" s="103"/>
-      <c r="H22" s="104"/>
+      <c r="G22" s="148"/>
+      <c r="H22" s="119"/>
       <c r="J22" s="38"/>
-      <c r="K22" s="144" t="s">
+      <c r="K22" s="150" t="s">
         <v>61</v>
       </c>
-      <c r="L22" s="97"/>
-      <c r="M22" s="97"/>
-      <c r="N22" s="98"/>
+      <c r="L22" s="103"/>
+      <c r="M22" s="103"/>
+      <c r="N22" s="104"/>
     </row>
     <row r="23" spans="1:14" ht="17.25" customHeight="1">
       <c r="B23" s="44"/>
       <c r="C23" s="44"/>
-      <c r="D23" s="105" t="s">
+      <c r="D23" s="141" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="104"/>
-      <c r="F23" s="104"/>
-      <c r="G23" s="104"/>
-      <c r="H23" s="104"/>
-      <c r="I23" s="104"/>
+      <c r="E23" s="119"/>
+      <c r="F23" s="119"/>
+      <c r="G23" s="119"/>
+      <c r="H23" s="119"/>
+      <c r="I23" s="119"/>
       <c r="J23" s="38"/>
-      <c r="K23" s="144" t="s">
+      <c r="K23" s="150" t="s">
         <v>62</v>
       </c>
-      <c r="L23" s="97"/>
-      <c r="M23" s="97"/>
-      <c r="N23" s="98"/>
+      <c r="L23" s="103"/>
+      <c r="M23" s="103"/>
+      <c r="N23" s="104"/>
     </row>
     <row r="24" spans="1:14" ht="13.5" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="44"/>
       <c r="C24" s="44"/>
-      <c r="D24" s="104"/>
-      <c r="E24" s="104"/>
-      <c r="F24" s="104"/>
-      <c r="G24" s="104"/>
-      <c r="H24" s="104"/>
-      <c r="I24" s="104"/>
+      <c r="D24" s="119"/>
+      <c r="E24" s="119"/>
+      <c r="F24" s="119"/>
+      <c r="G24" s="119"/>
+      <c r="H24" s="119"/>
+      <c r="I24" s="119"/>
       <c r="J24" s="40"/>
       <c r="K24" s="41" t="s">
         <v>63</v>
@@ -3640,19 +3723,19 @@
       <c r="A25" s="44"/>
       <c r="B25" s="44"/>
       <c r="C25" s="44"/>
-      <c r="D25" s="104"/>
-      <c r="E25" s="104"/>
-      <c r="F25" s="104"/>
-      <c r="G25" s="104"/>
-      <c r="H25" s="104"/>
-      <c r="I25" s="104"/>
+      <c r="D25" s="119"/>
+      <c r="E25" s="119"/>
+      <c r="F25" s="119"/>
+      <c r="G25" s="119"/>
+      <c r="H25" s="119"/>
+      <c r="I25" s="119"/>
       <c r="J25" s="38"/>
-      <c r="K25" s="144" t="s">
+      <c r="K25" s="150" t="s">
         <v>64</v>
       </c>
-      <c r="L25" s="97"/>
-      <c r="M25" s="97"/>
-      <c r="N25" s="98"/>
+      <c r="L25" s="103"/>
+      <c r="M25" s="103"/>
+      <c r="N25" s="104"/>
     </row>
     <row r="26" spans="1:14" ht="13.5" customHeight="1">
       <c r="J26" s="38"/>
@@ -3703,257 +3786,257 @@
       <c r="L28" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="M28" s="140" t="s">
+      <c r="M28" s="108" t="s">
         <v>46</v>
       </c>
-      <c r="N28" s="141"/>
+      <c r="N28" s="109"/>
     </row>
     <row r="29" spans="1:14" ht="13.5" customHeight="1">
       <c r="A29" s="65"/>
-      <c r="B29" s="127"/>
-      <c r="C29" s="128"/>
-      <c r="D29" s="128"/>
-      <c r="E29" s="128"/>
-      <c r="F29" s="128"/>
-      <c r="G29" s="128"/>
-      <c r="H29" s="128"/>
-      <c r="I29" s="129"/>
+      <c r="B29" s="121"/>
+      <c r="C29" s="122"/>
+      <c r="D29" s="122"/>
+      <c r="E29" s="122"/>
+      <c r="F29" s="122"/>
+      <c r="G29" s="122"/>
+      <c r="H29" s="122"/>
+      <c r="I29" s="123"/>
       <c r="J29" s="66"/>
       <c r="K29" s="67">
         <f t="shared" ref="K29:K41" si="0">A29*J29</f>
         <v>0</v>
       </c>
       <c r="L29" s="68"/>
-      <c r="M29" s="133"/>
-      <c r="N29" s="134"/>
+      <c r="M29" s="96"/>
+      <c r="N29" s="97"/>
     </row>
     <row r="30" spans="1:14" ht="13.5" customHeight="1">
       <c r="A30" s="69"/>
-      <c r="B30" s="96"/>
-      <c r="C30" s="97"/>
-      <c r="D30" s="97"/>
-      <c r="E30" s="97"/>
-      <c r="F30" s="97"/>
-      <c r="G30" s="97"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="98"/>
+      <c r="B30" s="124"/>
+      <c r="C30" s="103"/>
+      <c r="D30" s="103"/>
+      <c r="E30" s="103"/>
+      <c r="F30" s="103"/>
+      <c r="G30" s="103"/>
+      <c r="H30" s="103"/>
+      <c r="I30" s="104"/>
       <c r="J30" s="70"/>
       <c r="K30" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L30" s="72"/>
-      <c r="M30" s="118"/>
-      <c r="N30" s="119"/>
+      <c r="M30" s="98"/>
+      <c r="N30" s="99"/>
     </row>
     <row r="31" spans="1:14" ht="13.5" customHeight="1">
       <c r="A31" s="69"/>
-      <c r="B31" s="96"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="97"/>
-      <c r="E31" s="97"/>
-      <c r="F31" s="97"/>
-      <c r="G31" s="97"/>
-      <c r="H31" s="97"/>
-      <c r="I31" s="98"/>
+      <c r="B31" s="124"/>
+      <c r="C31" s="103"/>
+      <c r="D31" s="103"/>
+      <c r="E31" s="103"/>
+      <c r="F31" s="103"/>
+      <c r="G31" s="103"/>
+      <c r="H31" s="103"/>
+      <c r="I31" s="104"/>
       <c r="J31" s="73"/>
       <c r="K31" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L31" s="72"/>
-      <c r="M31" s="118"/>
-      <c r="N31" s="119"/>
+      <c r="M31" s="98"/>
+      <c r="N31" s="99"/>
     </row>
     <row r="32" spans="1:14" ht="13.5" customHeight="1">
       <c r="A32" s="69"/>
-      <c r="B32" s="96"/>
-      <c r="C32" s="97"/>
-      <c r="D32" s="97"/>
-      <c r="E32" s="97"/>
-      <c r="F32" s="97"/>
-      <c r="G32" s="97"/>
-      <c r="H32" s="97"/>
-      <c r="I32" s="98"/>
+      <c r="B32" s="124"/>
+      <c r="C32" s="103"/>
+      <c r="D32" s="103"/>
+      <c r="E32" s="103"/>
+      <c r="F32" s="103"/>
+      <c r="G32" s="103"/>
+      <c r="H32" s="103"/>
+      <c r="I32" s="104"/>
       <c r="J32" s="73"/>
       <c r="K32" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L32" s="72"/>
-      <c r="M32" s="118"/>
-      <c r="N32" s="119"/>
+      <c r="M32" s="98"/>
+      <c r="N32" s="99"/>
     </row>
     <row r="33" spans="1:14" ht="13.5" customHeight="1">
       <c r="A33" s="69"/>
-      <c r="B33" s="96"/>
-      <c r="C33" s="97"/>
-      <c r="D33" s="97"/>
-      <c r="E33" s="97"/>
-      <c r="F33" s="97"/>
-      <c r="G33" s="97"/>
-      <c r="H33" s="97"/>
-      <c r="I33" s="98"/>
+      <c r="B33" s="124"/>
+      <c r="C33" s="103"/>
+      <c r="D33" s="103"/>
+      <c r="E33" s="103"/>
+      <c r="F33" s="103"/>
+      <c r="G33" s="103"/>
+      <c r="H33" s="103"/>
+      <c r="I33" s="104"/>
       <c r="J33" s="73"/>
       <c r="K33" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L33" s="72"/>
-      <c r="M33" s="118"/>
-      <c r="N33" s="119"/>
+      <c r="M33" s="98"/>
+      <c r="N33" s="99"/>
     </row>
     <row r="34" spans="1:14" ht="13.5" customHeight="1">
       <c r="A34" s="69"/>
-      <c r="B34" s="96"/>
-      <c r="C34" s="97"/>
-      <c r="D34" s="97"/>
-      <c r="E34" s="97"/>
-      <c r="F34" s="97"/>
-      <c r="G34" s="97"/>
-      <c r="H34" s="97"/>
-      <c r="I34" s="98"/>
+      <c r="B34" s="124"/>
+      <c r="C34" s="103"/>
+      <c r="D34" s="103"/>
+      <c r="E34" s="103"/>
+      <c r="F34" s="103"/>
+      <c r="G34" s="103"/>
+      <c r="H34" s="103"/>
+      <c r="I34" s="104"/>
       <c r="J34" s="70"/>
       <c r="K34" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L34" s="72"/>
-      <c r="M34" s="118"/>
-      <c r="N34" s="119"/>
+      <c r="M34" s="98"/>
+      <c r="N34" s="99"/>
     </row>
     <row r="35" spans="1:14" ht="13.5" customHeight="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="96"/>
-      <c r="C35" s="97"/>
-      <c r="D35" s="97"/>
-      <c r="E35" s="97"/>
-      <c r="F35" s="97"/>
-      <c r="G35" s="97"/>
-      <c r="H35" s="97"/>
-      <c r="I35" s="98"/>
+      <c r="B35" s="124"/>
+      <c r="C35" s="103"/>
+      <c r="D35" s="103"/>
+      <c r="E35" s="103"/>
+      <c r="F35" s="103"/>
+      <c r="G35" s="103"/>
+      <c r="H35" s="103"/>
+      <c r="I35" s="104"/>
       <c r="J35" s="70"/>
       <c r="K35" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L35" s="72"/>
-      <c r="M35" s="118"/>
-      <c r="N35" s="119"/>
+      <c r="M35" s="98"/>
+      <c r="N35" s="99"/>
     </row>
     <row r="36" spans="1:14" ht="13.5" customHeight="1">
       <c r="A36" s="69"/>
-      <c r="B36" s="96"/>
-      <c r="C36" s="97"/>
-      <c r="D36" s="97"/>
-      <c r="E36" s="97"/>
-      <c r="F36" s="97"/>
-      <c r="G36" s="97"/>
-      <c r="H36" s="97"/>
-      <c r="I36" s="98"/>
+      <c r="B36" s="124"/>
+      <c r="C36" s="103"/>
+      <c r="D36" s="103"/>
+      <c r="E36" s="103"/>
+      <c r="F36" s="103"/>
+      <c r="G36" s="103"/>
+      <c r="H36" s="103"/>
+      <c r="I36" s="104"/>
       <c r="J36" s="70"/>
       <c r="K36" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L36" s="72"/>
-      <c r="M36" s="118"/>
-      <c r="N36" s="119"/>
+      <c r="M36" s="98"/>
+      <c r="N36" s="99"/>
     </row>
     <row r="37" spans="1:14" ht="13.5" customHeight="1">
       <c r="A37" s="69"/>
-      <c r="B37" s="96"/>
-      <c r="C37" s="97"/>
-      <c r="D37" s="97"/>
-      <c r="E37" s="97"/>
-      <c r="F37" s="97"/>
-      <c r="G37" s="97"/>
-      <c r="H37" s="97"/>
-      <c r="I37" s="98"/>
+      <c r="B37" s="124"/>
+      <c r="C37" s="103"/>
+      <c r="D37" s="103"/>
+      <c r="E37" s="103"/>
+      <c r="F37" s="103"/>
+      <c r="G37" s="103"/>
+      <c r="H37" s="103"/>
+      <c r="I37" s="104"/>
       <c r="J37" s="70"/>
       <c r="K37" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L37" s="72"/>
-      <c r="M37" s="118"/>
-      <c r="N37" s="119"/>
+      <c r="M37" s="98"/>
+      <c r="N37" s="99"/>
     </row>
     <row r="38" spans="1:14" ht="13.5" customHeight="1">
       <c r="A38" s="69"/>
-      <c r="B38" s="96"/>
-      <c r="C38" s="97"/>
-      <c r="D38" s="97"/>
-      <c r="E38" s="97"/>
-      <c r="F38" s="97"/>
-      <c r="G38" s="97"/>
-      <c r="H38" s="97"/>
-      <c r="I38" s="98"/>
+      <c r="B38" s="124"/>
+      <c r="C38" s="103"/>
+      <c r="D38" s="103"/>
+      <c r="E38" s="103"/>
+      <c r="F38" s="103"/>
+      <c r="G38" s="103"/>
+      <c r="H38" s="103"/>
+      <c r="I38" s="104"/>
       <c r="J38" s="70"/>
       <c r="K38" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L38" s="72"/>
-      <c r="M38" s="118"/>
-      <c r="N38" s="119"/>
+      <c r="M38" s="98"/>
+      <c r="N38" s="99"/>
     </row>
     <row r="39" spans="1:14" ht="13.5" customHeight="1">
       <c r="A39" s="69"/>
-      <c r="B39" s="96"/>
-      <c r="C39" s="97"/>
-      <c r="D39" s="97"/>
-      <c r="E39" s="97"/>
-      <c r="F39" s="97"/>
-      <c r="G39" s="97"/>
-      <c r="H39" s="97"/>
-      <c r="I39" s="98"/>
+      <c r="B39" s="124"/>
+      <c r="C39" s="103"/>
+      <c r="D39" s="103"/>
+      <c r="E39" s="103"/>
+      <c r="F39" s="103"/>
+      <c r="G39" s="103"/>
+      <c r="H39" s="103"/>
+      <c r="I39" s="104"/>
       <c r="J39" s="70"/>
       <c r="K39" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L39" s="72"/>
-      <c r="M39" s="118"/>
-      <c r="N39" s="119"/>
+      <c r="M39" s="98"/>
+      <c r="N39" s="99"/>
     </row>
     <row r="40" spans="1:14" ht="13.5" customHeight="1">
       <c r="A40" s="69"/>
-      <c r="B40" s="96"/>
-      <c r="C40" s="97"/>
-      <c r="D40" s="97"/>
-      <c r="E40" s="97"/>
-      <c r="F40" s="97"/>
-      <c r="G40" s="97"/>
-      <c r="H40" s="97"/>
-      <c r="I40" s="98"/>
+      <c r="B40" s="124"/>
+      <c r="C40" s="103"/>
+      <c r="D40" s="103"/>
+      <c r="E40" s="103"/>
+      <c r="F40" s="103"/>
+      <c r="G40" s="103"/>
+      <c r="H40" s="103"/>
+      <c r="I40" s="104"/>
       <c r="J40" s="70"/>
       <c r="K40" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L40" s="72"/>
-      <c r="M40" s="118"/>
-      <c r="N40" s="119"/>
+      <c r="M40" s="98"/>
+      <c r="N40" s="99"/>
     </row>
     <row r="41" spans="1:14" ht="13.5" customHeight="1">
       <c r="A41" s="74"/>
-      <c r="B41" s="130"/>
-      <c r="C41" s="131"/>
-      <c r="D41" s="131"/>
-      <c r="E41" s="131"/>
-      <c r="F41" s="131"/>
-      <c r="G41" s="131"/>
-      <c r="H41" s="131"/>
-      <c r="I41" s="132"/>
+      <c r="B41" s="125"/>
+      <c r="C41" s="126"/>
+      <c r="D41" s="126"/>
+      <c r="E41" s="126"/>
+      <c r="F41" s="126"/>
+      <c r="G41" s="126"/>
+      <c r="H41" s="126"/>
+      <c r="I41" s="127"/>
       <c r="J41" s="75"/>
       <c r="K41" s="76">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L41" s="77"/>
-      <c r="M41" s="116"/>
-      <c r="N41" s="117"/>
+      <c r="M41" s="110"/>
+      <c r="N41" s="111"/>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
       <c r="A42" s="78"/>
@@ -4076,32 +4159,20 @@
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A14:I14"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="D23:I25"/>
-    <mergeCell ref="M37:N37"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="M40:N40"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="M3:N4"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B35:I35"/>
     <mergeCell ref="M41:N41"/>
     <mergeCell ref="M35:N35"/>
     <mergeCell ref="D7:G7"/>
@@ -4118,20 +4189,32 @@
     <mergeCell ref="M30:N30"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="B39:I39"/>
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="M3:N4"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="M40:N40"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="D23:I25"/>
+    <mergeCell ref="M37:N37"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A9:I9"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A9">

</xml_diff>

<commit_message>
corrección en tipo de solicitud y plantilla
</commit_message>
<xml_diff>
--- a/netlify/functions/plantilla.xlsx
+++ b/netlify/functions/plantilla.xlsx
@@ -714,7 +714,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="53">
+  <fonts count="57">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1016,6 +1016,29 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF002060"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF002060"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="5.55"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="5.55"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1696,7 +1719,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="177">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1911,14 +1934,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="37" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="37" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="37" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1943,10 +2002,10 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1954,6 +2013,7 @@
     <xf numFmtId="20" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1977,6 +2037,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1986,12 +2049,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="52" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2003,9 +2066,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2024,6 +2084,20 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="45" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -2037,12 +2111,12 @@
     <xf numFmtId="14" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2446,13 +2520,13 @@
     <col min="4" max="4" width="5" customWidth="1"/>
     <col min="5" max="5" width="6" customWidth="1"/>
     <col min="6" max="6" width="4.109375" customWidth="1"/>
-    <col min="7" max="7" width="9.44140625" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
     <col min="8" max="8" width="6.44140625" customWidth="1"/>
     <col min="9" max="9" width="8.44140625" customWidth="1"/>
-    <col min="10" max="10" width="4.6640625" customWidth="1"/>
-    <col min="11" max="11" width="6.88671875" customWidth="1"/>
-    <col min="12" max="13" width="5.88671875" customWidth="1"/>
-    <col min="14" max="14" width="5.6640625" customWidth="1"/>
+    <col min="10" max="10" width="6.33203125" customWidth="1"/>
+    <col min="11" max="12" width="6.88671875" customWidth="1"/>
+    <col min="13" max="13" width="5.88671875" customWidth="1"/>
+    <col min="14" max="14" width="6.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="14.4">
@@ -2460,20 +2534,20 @@
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="128" t="s">
+      <c r="C1" s="142" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="125"/>
       <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="128"/>
-      <c r="I1" s="129"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="143"/>
       <c r="J1" s="4"/>
-      <c r="L1" s="130"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="113"/>
+      <c r="L1" s="144"/>
+      <c r="M1" s="125"/>
+      <c r="N1" s="125"/>
     </row>
     <row r="2" spans="1:14" ht="13.5" customHeight="1">
       <c r="A2" s="6"/>
@@ -2485,9 +2559,9 @@
         <v>3</v>
       </c>
       <c r="K2" s="8"/>
-      <c r="L2" s="131"/>
-      <c r="M2" s="132"/>
-      <c r="N2" s="132"/>
+      <c r="L2" s="145"/>
+      <c r="M2" s="146"/>
+      <c r="N2" s="146"/>
     </row>
     <row r="3" spans="1:14" ht="13.5" customHeight="1">
       <c r="A3" s="9" t="s">
@@ -2498,10 +2572,10 @@
         <v>5</v>
       </c>
       <c r="L3" s="10"/>
-      <c r="M3" s="133" t="s">
+      <c r="M3" s="147" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="134"/>
+      <c r="N3" s="148"/>
     </row>
     <row r="4" spans="1:14" ht="13.5" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -2516,12 +2590,12 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
       <c r="J4" s="11"/>
-      <c r="K4" s="154" t="s">
+      <c r="K4" s="96" t="s">
         <v>8</v>
       </c>
       <c r="L4" s="13"/>
-      <c r="M4" s="135"/>
-      <c r="N4" s="136"/>
+      <c r="M4" s="149"/>
+      <c r="N4" s="150"/>
     </row>
     <row r="5" spans="1:14" ht="13.5" customHeight="1">
       <c r="A5" s="9" t="s">
@@ -2530,11 +2604,11 @@
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="115"/>
-      <c r="F5" s="113"/>
-      <c r="G5" s="113"/>
-      <c r="H5" s="113"/>
-      <c r="I5" s="113"/>
+      <c r="E5" s="128"/>
+      <c r="F5" s="125"/>
+      <c r="G5" s="125"/>
+      <c r="H5" s="125"/>
+      <c r="I5" s="125"/>
       <c r="J5" s="4"/>
       <c r="K5" s="14" t="s">
         <v>10</v>
@@ -2550,15 +2624,15 @@
         <v>12</v>
       </c>
       <c r="B6" s="9"/>
-      <c r="C6" s="112"/>
-      <c r="D6" s="113"/>
-      <c r="E6" s="113"/>
-      <c r="F6" s="113"/>
+      <c r="C6" s="124"/>
+      <c r="D6" s="125"/>
+      <c r="E6" s="125"/>
+      <c r="F6" s="125"/>
       <c r="G6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="114"/>
-      <c r="I6" s="99"/>
+      <c r="H6" s="126"/>
+      <c r="I6" s="127"/>
       <c r="J6" s="4"/>
       <c r="K6" s="14" t="s">
         <v>14</v>
@@ -2575,10 +2649,10 @@
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="115"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="D7" s="128"/>
+      <c r="E7" s="125"/>
+      <c r="F7" s="125"/>
+      <c r="G7" s="125"/>
       <c r="H7" s="9" t="s">
         <v>17</v>
       </c>
@@ -2587,8 +2661,8 @@
       <c r="K7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="116"/>
-      <c r="M7" s="117"/>
+      <c r="L7" s="129"/>
+      <c r="M7" s="130"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:14" ht="13.5" customHeight="1">
@@ -2606,19 +2680,19 @@
         <v>21</v>
       </c>
       <c r="K8" s="21"/>
-      <c r="L8" s="120"/>
-      <c r="M8" s="103"/>
-      <c r="N8" s="103"/>
+      <c r="L8" s="133"/>
+      <c r="M8" s="115"/>
+      <c r="N8" s="115"/>
     </row>
     <row r="9" spans="1:14" ht="13.5" customHeight="1">
       <c r="A9" s="94" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="115"/>
-      <c r="D9" s="113"/>
-      <c r="E9" s="113"/>
-      <c r="F9" s="113"/>
-      <c r="G9" s="113"/>
+      <c r="C9" s="128"/>
+      <c r="D9" s="125"/>
+      <c r="E9" s="125"/>
+      <c r="F9" s="125"/>
+      <c r="G9" s="125"/>
       <c r="J9" s="22" t="s">
         <v>68</v>
       </c>
@@ -2655,40 +2729,40 @@
       <c r="N11" s="28"/>
     </row>
     <row r="12" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A12" s="137"/>
-      <c r="B12" s="137"/>
-      <c r="C12" s="137"/>
-      <c r="D12" s="137"/>
-      <c r="E12" s="137"/>
-      <c r="F12" s="137"/>
-      <c r="G12" s="137"/>
-      <c r="H12" s="137"/>
-      <c r="I12" s="138"/>
+      <c r="A12" s="151"/>
+      <c r="B12" s="151"/>
+      <c r="C12" s="151"/>
+      <c r="D12" s="151"/>
+      <c r="E12" s="151"/>
+      <c r="F12" s="151"/>
+      <c r="G12" s="151"/>
+      <c r="H12" s="151"/>
+      <c r="I12" s="152"/>
       <c r="J12" s="27"/>
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A13" s="137"/>
-      <c r="B13" s="137"/>
-      <c r="C13" s="137"/>
-      <c r="D13" s="137"/>
-      <c r="E13" s="137"/>
-      <c r="F13" s="137"/>
-      <c r="G13" s="137"/>
-      <c r="H13" s="137"/>
-      <c r="I13" s="138"/>
+      <c r="A13" s="151"/>
+      <c r="B13" s="151"/>
+      <c r="C13" s="151"/>
+      <c r="D13" s="151"/>
+      <c r="E13" s="151"/>
+      <c r="F13" s="151"/>
+      <c r="G13" s="151"/>
+      <c r="H13" s="151"/>
+      <c r="I13" s="152"/>
       <c r="J13" s="11"/>
     </row>
     <row r="14" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A14" s="137"/>
-      <c r="B14" s="137"/>
-      <c r="C14" s="137"/>
-      <c r="D14" s="137"/>
-      <c r="E14" s="137"/>
-      <c r="F14" s="137"/>
-      <c r="G14" s="137"/>
-      <c r="H14" s="137"/>
-      <c r="I14" s="138"/>
+      <c r="A14" s="151"/>
+      <c r="B14" s="151"/>
+      <c r="C14" s="151"/>
+      <c r="D14" s="151"/>
+      <c r="E14" s="151"/>
+      <c r="F14" s="151"/>
+      <c r="G14" s="151"/>
+      <c r="H14" s="151"/>
+      <c r="I14" s="152"/>
       <c r="J14" s="29"/>
       <c r="K14" s="6"/>
       <c r="L14" s="30"/>
@@ -2696,15 +2770,15 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A15" s="137"/>
-      <c r="B15" s="137"/>
-      <c r="C15" s="137"/>
-      <c r="D15" s="137"/>
-      <c r="E15" s="137"/>
-      <c r="F15" s="137"/>
-      <c r="G15" s="137"/>
-      <c r="H15" s="137"/>
-      <c r="I15" s="138"/>
+      <c r="A15" s="151"/>
+      <c r="B15" s="151"/>
+      <c r="C15" s="151"/>
+      <c r="D15" s="151"/>
+      <c r="E15" s="151"/>
+      <c r="F15" s="151"/>
+      <c r="G15" s="151"/>
+      <c r="H15" s="151"/>
+      <c r="I15" s="152"/>
       <c r="J15" s="29" t="s">
         <v>27</v>
       </c>
@@ -2714,15 +2788,15 @@
       <c r="N15" s="28"/>
     </row>
     <row r="16" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A16" s="137"/>
-      <c r="B16" s="137"/>
-      <c r="C16" s="137"/>
-      <c r="D16" s="137"/>
-      <c r="E16" s="137"/>
-      <c r="F16" s="137"/>
-      <c r="G16" s="137"/>
-      <c r="H16" s="137"/>
-      <c r="I16" s="138"/>
+      <c r="A16" s="151"/>
+      <c r="B16" s="151"/>
+      <c r="C16" s="151"/>
+      <c r="D16" s="151"/>
+      <c r="E16" s="151"/>
+      <c r="F16" s="151"/>
+      <c r="G16" s="151"/>
+      <c r="H16" s="151"/>
+      <c r="I16" s="152"/>
       <c r="J16" s="33" t="s">
         <v>28</v>
       </c>
@@ -2730,21 +2804,21 @@
         <v>66</v>
       </c>
       <c r="L16" s="35"/>
-      <c r="M16" s="100" t="s">
+      <c r="M16" s="112" t="s">
         <v>67</v>
       </c>
-      <c r="N16" s="101"/>
+      <c r="N16" s="113"/>
     </row>
     <row r="17" spans="1:14" ht="14.4">
-      <c r="A17" s="137"/>
-      <c r="B17" s="137"/>
-      <c r="C17" s="137"/>
-      <c r="D17" s="137"/>
-      <c r="E17" s="137"/>
-      <c r="F17" s="137"/>
-      <c r="G17" s="137"/>
-      <c r="H17" s="137"/>
-      <c r="I17" s="138"/>
+      <c r="A17" s="151"/>
+      <c r="B17" s="151"/>
+      <c r="C17" s="151"/>
+      <c r="D17" s="151"/>
+      <c r="E17" s="151"/>
+      <c r="F17" s="151"/>
+      <c r="G17" s="151"/>
+      <c r="H17" s="151"/>
+      <c r="I17" s="152"/>
       <c r="J17" s="36" t="s">
         <v>29</v>
       </c>
@@ -2754,28 +2828,28 @@
         <v>30</v>
       </c>
       <c r="J18" s="38"/>
-      <c r="K18" s="102" t="s">
+      <c r="K18" s="114" t="s">
         <v>31</v>
       </c>
-      <c r="L18" s="103"/>
-      <c r="M18" s="103"/>
-      <c r="N18" s="104"/>
+      <c r="L18" s="115"/>
+      <c r="M18" s="115"/>
+      <c r="N18" s="116"/>
     </row>
     <row r="19" spans="1:14" ht="13.5" customHeight="1">
       <c r="J19" s="38"/>
-      <c r="K19" s="102" t="s">
+      <c r="K19" s="114" t="s">
         <v>32</v>
       </c>
-      <c r="L19" s="103"/>
-      <c r="M19" s="103"/>
-      <c r="N19" s="104"/>
+      <c r="L19" s="115"/>
+      <c r="M19" s="115"/>
+      <c r="N19" s="116"/>
     </row>
     <row r="20" spans="1:14" ht="13.5" customHeight="1">
-      <c r="B20" s="118"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
+      <c r="B20" s="131"/>
+      <c r="C20" s="132"/>
+      <c r="D20" s="132"/>
+      <c r="E20" s="132"/>
+      <c r="F20" s="132"/>
       <c r="H20" s="39"/>
       <c r="J20" s="40"/>
       <c r="K20" s="41"/>
@@ -2790,58 +2864,58 @@
       <c r="D21" s="43"/>
       <c r="E21" s="26"/>
       <c r="J21" s="38"/>
-      <c r="K21" s="102" t="s">
+      <c r="K21" s="114" t="s">
         <v>34</v>
       </c>
-      <c r="L21" s="103"/>
-      <c r="M21" s="103"/>
-      <c r="N21" s="104"/>
+      <c r="L21" s="115"/>
+      <c r="M21" s="115"/>
+      <c r="N21" s="116"/>
     </row>
     <row r="22" spans="1:14" ht="23.25" customHeight="1">
       <c r="B22" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="142"/>
-      <c r="D22" s="142"/>
-      <c r="E22" s="142"/>
-      <c r="G22" s="139"/>
-      <c r="H22" s="140"/>
+      <c r="C22" s="155"/>
+      <c r="D22" s="155"/>
+      <c r="E22" s="155"/>
+      <c r="G22" s="153"/>
+      <c r="H22" s="154"/>
       <c r="J22" s="38"/>
-      <c r="K22" s="102" t="s">
+      <c r="K22" s="114" t="s">
         <v>36</v>
       </c>
-      <c r="L22" s="103"/>
-      <c r="M22" s="103"/>
-      <c r="N22" s="104"/>
+      <c r="L22" s="115"/>
+      <c r="M22" s="115"/>
+      <c r="N22" s="116"/>
     </row>
     <row r="23" spans="1:14" ht="17.25" customHeight="1">
       <c r="C23" s="44"/>
-      <c r="D23" s="155" t="s">
+      <c r="D23" s="141" t="s">
         <v>74</v>
       </c>
-      <c r="E23" s="155"/>
-      <c r="F23" s="155"/>
-      <c r="G23" s="155"/>
-      <c r="H23" s="155"/>
-      <c r="I23" s="155"/>
+      <c r="E23" s="141"/>
+      <c r="F23" s="141"/>
+      <c r="G23" s="141"/>
+      <c r="H23" s="141"/>
+      <c r="I23" s="141"/>
       <c r="J23" s="38"/>
-      <c r="K23" s="105" t="s">
+      <c r="K23" s="117" t="s">
         <v>38</v>
       </c>
-      <c r="L23" s="103"/>
-      <c r="M23" s="103"/>
-      <c r="N23" s="104"/>
+      <c r="L23" s="115"/>
+      <c r="M23" s="115"/>
+      <c r="N23" s="116"/>
     </row>
     <row r="24" spans="1:14" ht="13.5" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="44"/>
       <c r="C24" s="44"/>
-      <c r="D24" s="155"/>
-      <c r="E24" s="155"/>
-      <c r="F24" s="155"/>
-      <c r="G24" s="155"/>
-      <c r="H24" s="155"/>
-      <c r="I24" s="155"/>
+      <c r="D24" s="141"/>
+      <c r="E24" s="141"/>
+      <c r="F24" s="141"/>
+      <c r="G24" s="141"/>
+      <c r="H24" s="141"/>
+      <c r="I24" s="141"/>
       <c r="J24" s="40"/>
       <c r="K24" s="41"/>
       <c r="L24" s="42"/>
@@ -2852,25 +2926,25 @@
       <c r="A25" s="44"/>
       <c r="B25" s="44"/>
       <c r="C25" s="44"/>
-      <c r="D25" s="155"/>
-      <c r="E25" s="155"/>
-      <c r="F25" s="155"/>
-      <c r="G25" s="155"/>
-      <c r="H25" s="155"/>
-      <c r="I25" s="155"/>
+      <c r="D25" s="141"/>
+      <c r="E25" s="141"/>
+      <c r="F25" s="141"/>
+      <c r="G25" s="141"/>
+      <c r="H25" s="141"/>
+      <c r="I25" s="141"/>
       <c r="J25" s="38"/>
-      <c r="K25" s="105"/>
-      <c r="L25" s="106"/>
-      <c r="M25" s="106"/>
-      <c r="N25" s="107"/>
+      <c r="K25" s="117"/>
+      <c r="L25" s="118"/>
+      <c r="M25" s="118"/>
+      <c r="N25" s="119"/>
     </row>
     <row r="26" spans="1:14" ht="13.5" customHeight="1">
-      <c r="D26" s="155"/>
-      <c r="E26" s="155"/>
-      <c r="F26" s="155"/>
-      <c r="G26" s="155"/>
-      <c r="H26" s="155"/>
-      <c r="I26" s="155"/>
+      <c r="D26" s="141"/>
+      <c r="E26" s="141"/>
+      <c r="F26" s="141"/>
+      <c r="G26" s="141"/>
+      <c r="H26" s="141"/>
+      <c r="I26" s="141"/>
       <c r="J26" s="38"/>
       <c r="K26" s="45"/>
       <c r="L26" s="46"/>
@@ -2917,218 +2991,218 @@
       <c r="L28" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="M28" s="108" t="s">
+      <c r="M28" s="120" t="s">
         <v>46</v>
       </c>
-      <c r="N28" s="109"/>
+      <c r="N28" s="121"/>
     </row>
     <row r="29" spans="1:14" ht="13.5" customHeight="1">
       <c r="A29" s="65"/>
-      <c r="B29" s="121"/>
-      <c r="C29" s="122"/>
-      <c r="D29" s="122"/>
-      <c r="E29" s="122"/>
-      <c r="F29" s="122"/>
-      <c r="G29" s="122"/>
-      <c r="H29" s="122"/>
-      <c r="I29" s="123"/>
-      <c r="J29" s="66"/>
-      <c r="K29" s="67"/>
-      <c r="L29" s="68"/>
-      <c r="M29" s="96"/>
-      <c r="N29" s="97"/>
+      <c r="B29" s="134"/>
+      <c r="C29" s="135"/>
+      <c r="D29" s="135"/>
+      <c r="E29" s="135"/>
+      <c r="F29" s="135"/>
+      <c r="G29" s="135"/>
+      <c r="H29" s="135"/>
+      <c r="I29" s="136"/>
+      <c r="J29" s="98"/>
+      <c r="K29" s="99"/>
+      <c r="L29" s="100"/>
+      <c r="M29" s="108"/>
+      <c r="N29" s="109"/>
     </row>
     <row r="30" spans="1:14" ht="13.5" customHeight="1">
       <c r="A30" s="69"/>
-      <c r="B30" s="124"/>
-      <c r="C30" s="103"/>
-      <c r="D30" s="103"/>
-      <c r="E30" s="103"/>
-      <c r="F30" s="103"/>
-      <c r="G30" s="103"/>
-      <c r="H30" s="103"/>
-      <c r="I30" s="104"/>
-      <c r="J30" s="70"/>
-      <c r="K30" s="71"/>
-      <c r="L30" s="72"/>
-      <c r="M30" s="98"/>
-      <c r="N30" s="99"/>
+      <c r="B30" s="137"/>
+      <c r="C30" s="115"/>
+      <c r="D30" s="115"/>
+      <c r="E30" s="115"/>
+      <c r="F30" s="115"/>
+      <c r="G30" s="115"/>
+      <c r="H30" s="115"/>
+      <c r="I30" s="116"/>
+      <c r="J30" s="97"/>
+      <c r="K30" s="101"/>
+      <c r="L30" s="102"/>
+      <c r="M30" s="110"/>
+      <c r="N30" s="111"/>
     </row>
     <row r="31" spans="1:14" ht="13.5" customHeight="1">
       <c r="A31" s="69"/>
-      <c r="B31" s="124"/>
-      <c r="C31" s="103"/>
-      <c r="D31" s="103"/>
-      <c r="E31" s="103"/>
-      <c r="F31" s="103"/>
-      <c r="G31" s="103"/>
-      <c r="H31" s="103"/>
-      <c r="I31" s="104"/>
-      <c r="J31" s="73"/>
-      <c r="K31" s="71"/>
-      <c r="L31" s="72"/>
-      <c r="M31" s="98"/>
-      <c r="N31" s="99"/>
+      <c r="B31" s="137"/>
+      <c r="C31" s="115"/>
+      <c r="D31" s="115"/>
+      <c r="E31" s="115"/>
+      <c r="F31" s="115"/>
+      <c r="G31" s="115"/>
+      <c r="H31" s="115"/>
+      <c r="I31" s="116"/>
+      <c r="J31" s="97"/>
+      <c r="K31" s="101"/>
+      <c r="L31" s="102"/>
+      <c r="M31" s="110"/>
+      <c r="N31" s="111"/>
     </row>
     <row r="32" spans="1:14" ht="13.5" customHeight="1">
       <c r="A32" s="69"/>
-      <c r="B32" s="124"/>
-      <c r="C32" s="103"/>
-      <c r="D32" s="103"/>
-      <c r="E32" s="103"/>
-      <c r="F32" s="103"/>
-      <c r="G32" s="103"/>
-      <c r="H32" s="103"/>
-      <c r="I32" s="104"/>
-      <c r="J32" s="73"/>
-      <c r="K32" s="71"/>
-      <c r="L32" s="72"/>
-      <c r="M32" s="98"/>
-      <c r="N32" s="99"/>
+      <c r="B32" s="137"/>
+      <c r="C32" s="115"/>
+      <c r="D32" s="115"/>
+      <c r="E32" s="115"/>
+      <c r="F32" s="115"/>
+      <c r="G32" s="115"/>
+      <c r="H32" s="115"/>
+      <c r="I32" s="116"/>
+      <c r="J32" s="97"/>
+      <c r="K32" s="101"/>
+      <c r="L32" s="102"/>
+      <c r="M32" s="110"/>
+      <c r="N32" s="111"/>
     </row>
     <row r="33" spans="1:14" ht="13.5" customHeight="1">
       <c r="A33" s="69"/>
-      <c r="B33" s="124"/>
-      <c r="C33" s="103"/>
-      <c r="D33" s="103"/>
-      <c r="E33" s="103"/>
-      <c r="F33" s="103"/>
-      <c r="G33" s="103"/>
-      <c r="H33" s="103"/>
-      <c r="I33" s="104"/>
-      <c r="J33" s="73"/>
-      <c r="K33" s="71"/>
-      <c r="L33" s="72"/>
-      <c r="M33" s="98"/>
-      <c r="N33" s="99"/>
+      <c r="B33" s="137"/>
+      <c r="C33" s="115"/>
+      <c r="D33" s="115"/>
+      <c r="E33" s="115"/>
+      <c r="F33" s="115"/>
+      <c r="G33" s="115"/>
+      <c r="H33" s="115"/>
+      <c r="I33" s="116"/>
+      <c r="J33" s="97"/>
+      <c r="K33" s="101"/>
+      <c r="L33" s="102"/>
+      <c r="M33" s="110"/>
+      <c r="N33" s="111"/>
     </row>
     <row r="34" spans="1:14" ht="13.5" customHeight="1">
       <c r="A34" s="69"/>
-      <c r="B34" s="124"/>
-      <c r="C34" s="103"/>
-      <c r="D34" s="103"/>
-      <c r="E34" s="103"/>
-      <c r="F34" s="103"/>
-      <c r="G34" s="103"/>
-      <c r="H34" s="103"/>
-      <c r="I34" s="104"/>
-      <c r="J34" s="70"/>
-      <c r="K34" s="71"/>
-      <c r="L34" s="72"/>
-      <c r="M34" s="98"/>
-      <c r="N34" s="99"/>
+      <c r="B34" s="137"/>
+      <c r="C34" s="115"/>
+      <c r="D34" s="115"/>
+      <c r="E34" s="115"/>
+      <c r="F34" s="115"/>
+      <c r="G34" s="115"/>
+      <c r="H34" s="115"/>
+      <c r="I34" s="116"/>
+      <c r="J34" s="97"/>
+      <c r="K34" s="101"/>
+      <c r="L34" s="102"/>
+      <c r="M34" s="110"/>
+      <c r="N34" s="111"/>
     </row>
     <row r="35" spans="1:14" ht="13.5" customHeight="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="124"/>
-      <c r="C35" s="103"/>
-      <c r="D35" s="103"/>
-      <c r="E35" s="103"/>
-      <c r="F35" s="103"/>
-      <c r="G35" s="103"/>
-      <c r="H35" s="103"/>
-      <c r="I35" s="104"/>
-      <c r="J35" s="70"/>
-      <c r="K35" s="71"/>
-      <c r="L35" s="72"/>
-      <c r="M35" s="98"/>
-      <c r="N35" s="99"/>
+      <c r="B35" s="137"/>
+      <c r="C35" s="115"/>
+      <c r="D35" s="115"/>
+      <c r="E35" s="115"/>
+      <c r="F35" s="115"/>
+      <c r="G35" s="115"/>
+      <c r="H35" s="115"/>
+      <c r="I35" s="116"/>
+      <c r="J35" s="97"/>
+      <c r="K35" s="101"/>
+      <c r="L35" s="102"/>
+      <c r="M35" s="110"/>
+      <c r="N35" s="111"/>
     </row>
     <row r="36" spans="1:14" ht="13.5" customHeight="1">
       <c r="A36" s="69"/>
-      <c r="B36" s="124"/>
-      <c r="C36" s="103"/>
-      <c r="D36" s="103"/>
-      <c r="E36" s="103"/>
-      <c r="F36" s="103"/>
-      <c r="G36" s="103"/>
-      <c r="H36" s="103"/>
-      <c r="I36" s="104"/>
-      <c r="J36" s="70"/>
-      <c r="K36" s="71"/>
-      <c r="L36" s="72"/>
-      <c r="M36" s="98"/>
-      <c r="N36" s="99"/>
+      <c r="B36" s="137"/>
+      <c r="C36" s="115"/>
+      <c r="D36" s="115"/>
+      <c r="E36" s="115"/>
+      <c r="F36" s="115"/>
+      <c r="G36" s="115"/>
+      <c r="H36" s="115"/>
+      <c r="I36" s="116"/>
+      <c r="J36" s="97"/>
+      <c r="K36" s="101"/>
+      <c r="L36" s="102"/>
+      <c r="M36" s="110"/>
+      <c r="N36" s="111"/>
     </row>
     <row r="37" spans="1:14" ht="13.5" customHeight="1">
       <c r="A37" s="69"/>
-      <c r="B37" s="124"/>
-      <c r="C37" s="103"/>
-      <c r="D37" s="103"/>
-      <c r="E37" s="103"/>
-      <c r="F37" s="103"/>
-      <c r="G37" s="103"/>
-      <c r="H37" s="103"/>
-      <c r="I37" s="104"/>
-      <c r="J37" s="70"/>
-      <c r="K37" s="71"/>
-      <c r="L37" s="72"/>
-      <c r="M37" s="98"/>
-      <c r="N37" s="99"/>
+      <c r="B37" s="137"/>
+      <c r="C37" s="115"/>
+      <c r="D37" s="115"/>
+      <c r="E37" s="115"/>
+      <c r="F37" s="115"/>
+      <c r="G37" s="115"/>
+      <c r="H37" s="115"/>
+      <c r="I37" s="116"/>
+      <c r="J37" s="97"/>
+      <c r="K37" s="101"/>
+      <c r="L37" s="102"/>
+      <c r="M37" s="110"/>
+      <c r="N37" s="111"/>
     </row>
     <row r="38" spans="1:14" ht="13.5" customHeight="1">
       <c r="A38" s="69"/>
-      <c r="B38" s="124"/>
-      <c r="C38" s="103"/>
-      <c r="D38" s="103"/>
-      <c r="E38" s="103"/>
-      <c r="F38" s="103"/>
-      <c r="G38" s="103"/>
-      <c r="H38" s="103"/>
-      <c r="I38" s="104"/>
-      <c r="J38" s="70"/>
-      <c r="K38" s="71"/>
-      <c r="L38" s="72"/>
-      <c r="M38" s="98"/>
-      <c r="N38" s="99"/>
+      <c r="B38" s="137"/>
+      <c r="C38" s="115"/>
+      <c r="D38" s="115"/>
+      <c r="E38" s="115"/>
+      <c r="F38" s="115"/>
+      <c r="G38" s="115"/>
+      <c r="H38" s="115"/>
+      <c r="I38" s="116"/>
+      <c r="J38" s="97"/>
+      <c r="K38" s="101"/>
+      <c r="L38" s="102"/>
+      <c r="M38" s="110"/>
+      <c r="N38" s="111"/>
     </row>
     <row r="39" spans="1:14" ht="13.5" customHeight="1">
       <c r="A39" s="69"/>
-      <c r="B39" s="124"/>
-      <c r="C39" s="103"/>
-      <c r="D39" s="103"/>
-      <c r="E39" s="103"/>
-      <c r="F39" s="103"/>
-      <c r="G39" s="103"/>
-      <c r="H39" s="103"/>
-      <c r="I39" s="104"/>
-      <c r="J39" s="70"/>
-      <c r="K39" s="71"/>
-      <c r="L39" s="72"/>
-      <c r="M39" s="98"/>
-      <c r="N39" s="99"/>
+      <c r="B39" s="137"/>
+      <c r="C39" s="115"/>
+      <c r="D39" s="115"/>
+      <c r="E39" s="115"/>
+      <c r="F39" s="115"/>
+      <c r="G39" s="115"/>
+      <c r="H39" s="115"/>
+      <c r="I39" s="116"/>
+      <c r="J39" s="97"/>
+      <c r="K39" s="101"/>
+      <c r="L39" s="102"/>
+      <c r="M39" s="110"/>
+      <c r="N39" s="111"/>
     </row>
     <row r="40" spans="1:14" ht="13.5" customHeight="1">
       <c r="A40" s="69"/>
-      <c r="B40" s="124"/>
-      <c r="C40" s="103"/>
-      <c r="D40" s="103"/>
-      <c r="E40" s="103"/>
-      <c r="F40" s="103"/>
-      <c r="G40" s="103"/>
-      <c r="H40" s="103"/>
-      <c r="I40" s="104"/>
-      <c r="J40" s="70"/>
-      <c r="K40" s="71"/>
-      <c r="L40" s="72"/>
-      <c r="M40" s="98"/>
-      <c r="N40" s="99"/>
+      <c r="B40" s="137"/>
+      <c r="C40" s="115"/>
+      <c r="D40" s="115"/>
+      <c r="E40" s="115"/>
+      <c r="F40" s="115"/>
+      <c r="G40" s="115"/>
+      <c r="H40" s="115"/>
+      <c r="I40" s="116"/>
+      <c r="J40" s="97"/>
+      <c r="K40" s="101"/>
+      <c r="L40" s="102"/>
+      <c r="M40" s="110"/>
+      <c r="N40" s="111"/>
     </row>
     <row r="41" spans="1:14" ht="13.5" customHeight="1">
       <c r="A41" s="74"/>
-      <c r="B41" s="125"/>
-      <c r="C41" s="126"/>
-      <c r="D41" s="126"/>
-      <c r="E41" s="126"/>
-      <c r="F41" s="126"/>
-      <c r="G41" s="126"/>
-      <c r="H41" s="126"/>
-      <c r="I41" s="127"/>
-      <c r="J41" s="75"/>
-      <c r="K41" s="76"/>
-      <c r="L41" s="77"/>
-      <c r="M41" s="110"/>
-      <c r="N41" s="111"/>
+      <c r="B41" s="138"/>
+      <c r="C41" s="139"/>
+      <c r="D41" s="139"/>
+      <c r="E41" s="139"/>
+      <c r="F41" s="139"/>
+      <c r="G41" s="139"/>
+      <c r="H41" s="139"/>
+      <c r="I41" s="140"/>
+      <c r="J41" s="107"/>
+      <c r="K41" s="103"/>
+      <c r="L41" s="104"/>
+      <c r="M41" s="122"/>
+      <c r="N41" s="123"/>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
       <c r="A42" s="78"/>
@@ -3142,8 +3216,8 @@
       <c r="J42" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="K42" s="82"/>
-      <c r="L42" s="83" t="str">
+      <c r="K42" s="105"/>
+      <c r="L42" s="106" t="str">
         <f>IF(SUM(L29:L41)&gt;0,SUM(L29:L41),".")</f>
         <v>.</v>
       </c>
@@ -3235,17 +3309,17 @@
     <mergeCell ref="B34:I34"/>
     <mergeCell ref="B35:I35"/>
     <mergeCell ref="B36:I36"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A12:I17"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="C22:E22"/>
     <mergeCell ref="D23:I26"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="L1:N1"/>
     <mergeCell ref="L2:N2"/>
     <mergeCell ref="M3:N4"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A12:I17"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="C22:E22"/>
     <mergeCell ref="M41:N41"/>
     <mergeCell ref="M40:N40"/>
     <mergeCell ref="C6:F6"/>
@@ -3291,7 +3365,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.86614173228346458" right="0.39370078740157483" top="1.1811023622047245" bottom="0.39370078740157483" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="95" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C* Formulario de Solicitud y Aprobacion de Pago *</oddHeader>
     <oddFooter>&amp;R00-024βэηяμ</oddFooter>
@@ -3324,21 +3398,21 @@
         <v>54</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="128"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
+      <c r="C1" s="142"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="125"/>
       <c r="G1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="128"/>
-      <c r="I1" s="129"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="143"/>
       <c r="J1" s="4"/>
       <c r="K1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="130"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="113"/>
+      <c r="L1" s="144"/>
+      <c r="M1" s="125"/>
+      <c r="N1" s="125"/>
     </row>
     <row r="2" spans="1:14" ht="13.5" customHeight="1">
       <c r="A2" s="6"/>
@@ -3350,9 +3424,9 @@
         <v>3</v>
       </c>
       <c r="K2" s="8"/>
-      <c r="L2" s="153"/>
-      <c r="M2" s="103"/>
-      <c r="N2" s="103"/>
+      <c r="L2" s="172"/>
+      <c r="M2" s="115"/>
+      <c r="N2" s="115"/>
     </row>
     <row r="3" spans="1:14" ht="13.5" customHeight="1">
       <c r="A3" s="9" t="s">
@@ -3363,10 +3437,10 @@
         <v>5</v>
       </c>
       <c r="L3" s="10"/>
-      <c r="M3" s="133" t="s">
+      <c r="M3" s="173" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="134"/>
+      <c r="N3" s="174"/>
     </row>
     <row r="4" spans="1:14" ht="13.5" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -3385,8 +3459,8 @@
         <v>8</v>
       </c>
       <c r="L4" s="13"/>
-      <c r="M4" s="135"/>
-      <c r="N4" s="136"/>
+      <c r="M4" s="175"/>
+      <c r="N4" s="176"/>
     </row>
     <row r="5" spans="1:14" ht="13.5" customHeight="1">
       <c r="A5" s="9" t="s">
@@ -3395,11 +3469,11 @@
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
-      <c r="E5" s="115"/>
-      <c r="F5" s="113"/>
-      <c r="G5" s="113"/>
-      <c r="H5" s="113"/>
-      <c r="I5" s="113"/>
+      <c r="E5" s="128"/>
+      <c r="F5" s="125"/>
+      <c r="G5" s="125"/>
+      <c r="H5" s="125"/>
+      <c r="I5" s="125"/>
       <c r="J5" s="4"/>
       <c r="K5" s="14" t="s">
         <v>10</v>
@@ -3415,15 +3489,15 @@
         <v>12</v>
       </c>
       <c r="B6" s="9"/>
-      <c r="C6" s="112"/>
-      <c r="D6" s="113"/>
-      <c r="E6" s="113"/>
-      <c r="F6" s="113"/>
+      <c r="C6" s="124"/>
+      <c r="D6" s="125"/>
+      <c r="E6" s="125"/>
+      <c r="F6" s="125"/>
       <c r="G6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="114"/>
-      <c r="I6" s="99"/>
+      <c r="H6" s="126"/>
+      <c r="I6" s="127"/>
       <c r="J6" s="4"/>
       <c r="K6" s="14" t="s">
         <v>14</v>
@@ -3440,10 +3514,10 @@
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="115"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="D7" s="128"/>
+      <c r="E7" s="125"/>
+      <c r="F7" s="125"/>
+      <c r="G7" s="125"/>
       <c r="H7" s="9" t="s">
         <v>17</v>
       </c>
@@ -3452,11 +3526,11 @@
       <c r="K7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="149">
+      <c r="L7" s="168">
         <f>SUM(L4:L6)+N5+N6</f>
         <v>0</v>
       </c>
-      <c r="M7" s="117"/>
+      <c r="M7" s="130"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:14" ht="13.5" customHeight="1">
@@ -3474,22 +3548,22 @@
         <v>21</v>
       </c>
       <c r="K8" s="21"/>
-      <c r="L8" s="120"/>
-      <c r="M8" s="103"/>
-      <c r="N8" s="103"/>
+      <c r="L8" s="133"/>
+      <c r="M8" s="115"/>
+      <c r="N8" s="115"/>
     </row>
     <row r="9" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A9" s="146" t="s">
+      <c r="A9" s="159" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="119"/>
-      <c r="C9" s="119"/>
-      <c r="D9" s="119"/>
-      <c r="E9" s="119"/>
-      <c r="F9" s="119"/>
-      <c r="G9" s="119"/>
-      <c r="H9" s="119"/>
-      <c r="I9" s="147"/>
+      <c r="B9" s="132"/>
+      <c r="C9" s="132"/>
+      <c r="D9" s="132"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="132"/>
+      <c r="G9" s="132"/>
+      <c r="H9" s="132"/>
+      <c r="I9" s="160"/>
       <c r="J9" s="22" t="s">
         <v>23</v>
       </c>
@@ -3524,40 +3598,40 @@
       <c r="N11" s="28"/>
     </row>
     <row r="12" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A12" s="143"/>
-      <c r="B12" s="113"/>
-      <c r="C12" s="113"/>
-      <c r="D12" s="113"/>
-      <c r="E12" s="113"/>
-      <c r="F12" s="113"/>
-      <c r="G12" s="113"/>
-      <c r="H12" s="113"/>
-      <c r="I12" s="129"/>
+      <c r="A12" s="156"/>
+      <c r="B12" s="125"/>
+      <c r="C12" s="125"/>
+      <c r="D12" s="125"/>
+      <c r="E12" s="125"/>
+      <c r="F12" s="125"/>
+      <c r="G12" s="125"/>
+      <c r="H12" s="125"/>
+      <c r="I12" s="143"/>
       <c r="J12" s="27"/>
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A13" s="144"/>
-      <c r="B13" s="103"/>
-      <c r="C13" s="103"/>
-      <c r="D13" s="103"/>
-      <c r="E13" s="103"/>
-      <c r="F13" s="103"/>
-      <c r="G13" s="103"/>
-      <c r="H13" s="103"/>
-      <c r="I13" s="99"/>
+      <c r="A13" s="157"/>
+      <c r="B13" s="115"/>
+      <c r="C13" s="115"/>
+      <c r="D13" s="115"/>
+      <c r="E13" s="115"/>
+      <c r="F13" s="115"/>
+      <c r="G13" s="115"/>
+      <c r="H13" s="115"/>
+      <c r="I13" s="127"/>
       <c r="J13" s="11"/>
     </row>
     <row r="14" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A14" s="144"/>
-      <c r="B14" s="103"/>
-      <c r="C14" s="103"/>
-      <c r="D14" s="103"/>
-      <c r="E14" s="103"/>
-      <c r="F14" s="103"/>
-      <c r="G14" s="103"/>
-      <c r="H14" s="103"/>
-      <c r="I14" s="99"/>
+      <c r="A14" s="157"/>
+      <c r="B14" s="115"/>
+      <c r="C14" s="115"/>
+      <c r="D14" s="115"/>
+      <c r="E14" s="115"/>
+      <c r="F14" s="115"/>
+      <c r="G14" s="115"/>
+      <c r="H14" s="115"/>
+      <c r="I14" s="127"/>
       <c r="J14" s="29"/>
       <c r="K14" s="6"/>
       <c r="L14" s="30"/>
@@ -3565,15 +3639,15 @@
       <c r="N14" s="31"/>
     </row>
     <row r="15" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A15" s="144"/>
-      <c r="B15" s="103"/>
-      <c r="C15" s="103"/>
-      <c r="D15" s="103"/>
-      <c r="E15" s="103"/>
-      <c r="F15" s="103"/>
-      <c r="G15" s="103"/>
-      <c r="H15" s="103"/>
-      <c r="I15" s="99"/>
+      <c r="A15" s="157"/>
+      <c r="B15" s="115"/>
+      <c r="C15" s="115"/>
+      <c r="D15" s="115"/>
+      <c r="E15" s="115"/>
+      <c r="F15" s="115"/>
+      <c r="G15" s="115"/>
+      <c r="H15" s="115"/>
+      <c r="I15" s="127"/>
       <c r="J15" s="29" t="s">
         <v>55</v>
       </c>
@@ -3584,33 +3658,33 @@
       <c r="N15" s="28"/>
     </row>
     <row r="16" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A16" s="144"/>
-      <c r="B16" s="103"/>
-      <c r="C16" s="103"/>
-      <c r="D16" s="103"/>
-      <c r="E16" s="103"/>
-      <c r="F16" s="103"/>
-      <c r="G16" s="103"/>
-      <c r="H16" s="103"/>
-      <c r="I16" s="99"/>
+      <c r="A16" s="157"/>
+      <c r="B16" s="115"/>
+      <c r="C16" s="115"/>
+      <c r="D16" s="115"/>
+      <c r="E16" s="115"/>
+      <c r="F16" s="115"/>
+      <c r="G16" s="115"/>
+      <c r="H16" s="115"/>
+      <c r="I16" s="127"/>
       <c r="J16" s="33" t="s">
         <v>28</v>
       </c>
       <c r="K16" s="34"/>
       <c r="L16" s="35"/>
-      <c r="M16" s="151"/>
-      <c r="N16" s="152"/>
+      <c r="M16" s="170"/>
+      <c r="N16" s="171"/>
     </row>
     <row r="17" spans="1:14" ht="14.4">
-      <c r="A17" s="145"/>
-      <c r="B17" s="119"/>
-      <c r="C17" s="119"/>
-      <c r="D17" s="119"/>
-      <c r="E17" s="119"/>
-      <c r="F17" s="119"/>
-      <c r="G17" s="119"/>
-      <c r="H17" s="119"/>
-      <c r="I17" s="119"/>
+      <c r="A17" s="158"/>
+      <c r="B17" s="132"/>
+      <c r="C17" s="132"/>
+      <c r="D17" s="132"/>
+      <c r="E17" s="132"/>
+      <c r="F17" s="132"/>
+      <c r="G17" s="132"/>
+      <c r="H17" s="132"/>
+      <c r="I17" s="132"/>
       <c r="J17" s="36" t="s">
         <v>29</v>
       </c>
@@ -3620,28 +3694,28 @@
         <v>30</v>
       </c>
       <c r="J18" s="38"/>
-      <c r="K18" s="150" t="s">
+      <c r="K18" s="169" t="s">
         <v>57</v>
       </c>
-      <c r="L18" s="103"/>
-      <c r="M18" s="103"/>
-      <c r="N18" s="104"/>
+      <c r="L18" s="115"/>
+      <c r="M18" s="115"/>
+      <c r="N18" s="116"/>
     </row>
     <row r="19" spans="1:14" ht="13.5" customHeight="1">
       <c r="J19" s="38"/>
-      <c r="K19" s="150" t="s">
+      <c r="K19" s="169" t="s">
         <v>58</v>
       </c>
-      <c r="L19" s="103"/>
-      <c r="M19" s="103"/>
-      <c r="N19" s="104"/>
+      <c r="L19" s="115"/>
+      <c r="M19" s="115"/>
+      <c r="N19" s="116"/>
     </row>
     <row r="20" spans="1:14" ht="13.5" customHeight="1">
-      <c r="B20" s="118"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
+      <c r="B20" s="131"/>
+      <c r="C20" s="132"/>
+      <c r="D20" s="132"/>
+      <c r="E20" s="132"/>
+      <c r="F20" s="132"/>
       <c r="H20" s="39"/>
       <c r="J20" s="40"/>
       <c r="K20" s="41" t="s">
@@ -3658,59 +3732,59 @@
       <c r="D21" s="43"/>
       <c r="E21" s="26"/>
       <c r="J21" s="38"/>
-      <c r="K21" s="150" t="s">
+      <c r="K21" s="169" t="s">
         <v>60</v>
       </c>
-      <c r="L21" s="103"/>
-      <c r="M21" s="103"/>
-      <c r="N21" s="104"/>
+      <c r="L21" s="115"/>
+      <c r="M21" s="115"/>
+      <c r="N21" s="116"/>
     </row>
     <row r="22" spans="1:14" ht="17.25" customHeight="1">
       <c r="C22" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D22" s="142"/>
-      <c r="E22" s="119"/>
+      <c r="D22" s="155"/>
+      <c r="E22" s="132"/>
       <c r="F22" s="26"/>
-      <c r="G22" s="148"/>
-      <c r="H22" s="119"/>
+      <c r="G22" s="161"/>
+      <c r="H22" s="132"/>
       <c r="J22" s="38"/>
-      <c r="K22" s="150" t="s">
+      <c r="K22" s="169" t="s">
         <v>61</v>
       </c>
-      <c r="L22" s="103"/>
-      <c r="M22" s="103"/>
-      <c r="N22" s="104"/>
+      <c r="L22" s="115"/>
+      <c r="M22" s="115"/>
+      <c r="N22" s="116"/>
     </row>
     <row r="23" spans="1:14" ht="17.25" customHeight="1">
       <c r="B23" s="44"/>
       <c r="C23" s="44"/>
-      <c r="D23" s="141" t="s">
+      <c r="D23" s="162" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="119"/>
-      <c r="F23" s="119"/>
-      <c r="G23" s="119"/>
-      <c r="H23" s="119"/>
-      <c r="I23" s="119"/>
+      <c r="E23" s="132"/>
+      <c r="F23" s="132"/>
+      <c r="G23" s="132"/>
+      <c r="H23" s="132"/>
+      <c r="I23" s="132"/>
       <c r="J23" s="38"/>
-      <c r="K23" s="150" t="s">
+      <c r="K23" s="169" t="s">
         <v>62</v>
       </c>
-      <c r="L23" s="103"/>
-      <c r="M23" s="103"/>
-      <c r="N23" s="104"/>
+      <c r="L23" s="115"/>
+      <c r="M23" s="115"/>
+      <c r="N23" s="116"/>
     </row>
     <row r="24" spans="1:14" ht="13.5" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="44"/>
       <c r="C24" s="44"/>
-      <c r="D24" s="119"/>
-      <c r="E24" s="119"/>
-      <c r="F24" s="119"/>
-      <c r="G24" s="119"/>
-      <c r="H24" s="119"/>
-      <c r="I24" s="119"/>
+      <c r="D24" s="132"/>
+      <c r="E24" s="132"/>
+      <c r="F24" s="132"/>
+      <c r="G24" s="132"/>
+      <c r="H24" s="132"/>
+      <c r="I24" s="132"/>
       <c r="J24" s="40"/>
       <c r="K24" s="41" t="s">
         <v>63</v>
@@ -3723,19 +3797,19 @@
       <c r="A25" s="44"/>
       <c r="B25" s="44"/>
       <c r="C25" s="44"/>
-      <c r="D25" s="119"/>
-      <c r="E25" s="119"/>
-      <c r="F25" s="119"/>
-      <c r="G25" s="119"/>
-      <c r="H25" s="119"/>
-      <c r="I25" s="119"/>
+      <c r="D25" s="132"/>
+      <c r="E25" s="132"/>
+      <c r="F25" s="132"/>
+      <c r="G25" s="132"/>
+      <c r="H25" s="132"/>
+      <c r="I25" s="132"/>
       <c r="J25" s="38"/>
-      <c r="K25" s="150" t="s">
+      <c r="K25" s="169" t="s">
         <v>64</v>
       </c>
-      <c r="L25" s="103"/>
-      <c r="M25" s="103"/>
-      <c r="N25" s="104"/>
+      <c r="L25" s="115"/>
+      <c r="M25" s="115"/>
+      <c r="N25" s="116"/>
     </row>
     <row r="26" spans="1:14" ht="13.5" customHeight="1">
       <c r="J26" s="38"/>
@@ -3786,257 +3860,257 @@
       <c r="L28" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="M28" s="108" t="s">
+      <c r="M28" s="120" t="s">
         <v>46</v>
       </c>
-      <c r="N28" s="109"/>
+      <c r="N28" s="121"/>
     </row>
     <row r="29" spans="1:14" ht="13.5" customHeight="1">
       <c r="A29" s="65"/>
-      <c r="B29" s="121"/>
-      <c r="C29" s="122"/>
-      <c r="D29" s="122"/>
-      <c r="E29" s="122"/>
-      <c r="F29" s="122"/>
-      <c r="G29" s="122"/>
-      <c r="H29" s="122"/>
-      <c r="I29" s="123"/>
+      <c r="B29" s="134"/>
+      <c r="C29" s="135"/>
+      <c r="D29" s="135"/>
+      <c r="E29" s="135"/>
+      <c r="F29" s="135"/>
+      <c r="G29" s="135"/>
+      <c r="H29" s="135"/>
+      <c r="I29" s="136"/>
       <c r="J29" s="66"/>
       <c r="K29" s="67">
         <f t="shared" ref="K29:K41" si="0">A29*J29</f>
         <v>0</v>
       </c>
       <c r="L29" s="68"/>
-      <c r="M29" s="96"/>
-      <c r="N29" s="97"/>
+      <c r="M29" s="164"/>
+      <c r="N29" s="165"/>
     </row>
     <row r="30" spans="1:14" ht="13.5" customHeight="1">
       <c r="A30" s="69"/>
-      <c r="B30" s="124"/>
-      <c r="C30" s="103"/>
-      <c r="D30" s="103"/>
-      <c r="E30" s="103"/>
-      <c r="F30" s="103"/>
-      <c r="G30" s="103"/>
-      <c r="H30" s="103"/>
-      <c r="I30" s="104"/>
+      <c r="B30" s="137"/>
+      <c r="C30" s="115"/>
+      <c r="D30" s="115"/>
+      <c r="E30" s="115"/>
+      <c r="F30" s="115"/>
+      <c r="G30" s="115"/>
+      <c r="H30" s="115"/>
+      <c r="I30" s="116"/>
       <c r="J30" s="70"/>
       <c r="K30" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L30" s="72"/>
-      <c r="M30" s="98"/>
-      <c r="N30" s="99"/>
+      <c r="M30" s="163"/>
+      <c r="N30" s="127"/>
     </row>
     <row r="31" spans="1:14" ht="13.5" customHeight="1">
       <c r="A31" s="69"/>
-      <c r="B31" s="124"/>
-      <c r="C31" s="103"/>
-      <c r="D31" s="103"/>
-      <c r="E31" s="103"/>
-      <c r="F31" s="103"/>
-      <c r="G31" s="103"/>
-      <c r="H31" s="103"/>
-      <c r="I31" s="104"/>
+      <c r="B31" s="137"/>
+      <c r="C31" s="115"/>
+      <c r="D31" s="115"/>
+      <c r="E31" s="115"/>
+      <c r="F31" s="115"/>
+      <c r="G31" s="115"/>
+      <c r="H31" s="115"/>
+      <c r="I31" s="116"/>
       <c r="J31" s="73"/>
       <c r="K31" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L31" s="72"/>
-      <c r="M31" s="98"/>
-      <c r="N31" s="99"/>
+      <c r="M31" s="163"/>
+      <c r="N31" s="127"/>
     </row>
     <row r="32" spans="1:14" ht="13.5" customHeight="1">
       <c r="A32" s="69"/>
-      <c r="B32" s="124"/>
-      <c r="C32" s="103"/>
-      <c r="D32" s="103"/>
-      <c r="E32" s="103"/>
-      <c r="F32" s="103"/>
-      <c r="G32" s="103"/>
-      <c r="H32" s="103"/>
-      <c r="I32" s="104"/>
+      <c r="B32" s="137"/>
+      <c r="C32" s="115"/>
+      <c r="D32" s="115"/>
+      <c r="E32" s="115"/>
+      <c r="F32" s="115"/>
+      <c r="G32" s="115"/>
+      <c r="H32" s="115"/>
+      <c r="I32" s="116"/>
       <c r="J32" s="73"/>
       <c r="K32" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L32" s="72"/>
-      <c r="M32" s="98"/>
-      <c r="N32" s="99"/>
+      <c r="M32" s="163"/>
+      <c r="N32" s="127"/>
     </row>
     <row r="33" spans="1:14" ht="13.5" customHeight="1">
       <c r="A33" s="69"/>
-      <c r="B33" s="124"/>
-      <c r="C33" s="103"/>
-      <c r="D33" s="103"/>
-      <c r="E33" s="103"/>
-      <c r="F33" s="103"/>
-      <c r="G33" s="103"/>
-      <c r="H33" s="103"/>
-      <c r="I33" s="104"/>
+      <c r="B33" s="137"/>
+      <c r="C33" s="115"/>
+      <c r="D33" s="115"/>
+      <c r="E33" s="115"/>
+      <c r="F33" s="115"/>
+      <c r="G33" s="115"/>
+      <c r="H33" s="115"/>
+      <c r="I33" s="116"/>
       <c r="J33" s="73"/>
       <c r="K33" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L33" s="72"/>
-      <c r="M33" s="98"/>
-      <c r="N33" s="99"/>
+      <c r="M33" s="163"/>
+      <c r="N33" s="127"/>
     </row>
     <row r="34" spans="1:14" ht="13.5" customHeight="1">
       <c r="A34" s="69"/>
-      <c r="B34" s="124"/>
-      <c r="C34" s="103"/>
-      <c r="D34" s="103"/>
-      <c r="E34" s="103"/>
-      <c r="F34" s="103"/>
-      <c r="G34" s="103"/>
-      <c r="H34" s="103"/>
-      <c r="I34" s="104"/>
+      <c r="B34" s="137"/>
+      <c r="C34" s="115"/>
+      <c r="D34" s="115"/>
+      <c r="E34" s="115"/>
+      <c r="F34" s="115"/>
+      <c r="G34" s="115"/>
+      <c r="H34" s="115"/>
+      <c r="I34" s="116"/>
       <c r="J34" s="70"/>
       <c r="K34" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L34" s="72"/>
-      <c r="M34" s="98"/>
-      <c r="N34" s="99"/>
+      <c r="M34" s="163"/>
+      <c r="N34" s="127"/>
     </row>
     <row r="35" spans="1:14" ht="13.5" customHeight="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="124"/>
-      <c r="C35" s="103"/>
-      <c r="D35" s="103"/>
-      <c r="E35" s="103"/>
-      <c r="F35" s="103"/>
-      <c r="G35" s="103"/>
-      <c r="H35" s="103"/>
-      <c r="I35" s="104"/>
+      <c r="B35" s="137"/>
+      <c r="C35" s="115"/>
+      <c r="D35" s="115"/>
+      <c r="E35" s="115"/>
+      <c r="F35" s="115"/>
+      <c r="G35" s="115"/>
+      <c r="H35" s="115"/>
+      <c r="I35" s="116"/>
       <c r="J35" s="70"/>
       <c r="K35" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L35" s="72"/>
-      <c r="M35" s="98"/>
-      <c r="N35" s="99"/>
+      <c r="M35" s="163"/>
+      <c r="N35" s="127"/>
     </row>
     <row r="36" spans="1:14" ht="13.5" customHeight="1">
       <c r="A36" s="69"/>
-      <c r="B36" s="124"/>
-      <c r="C36" s="103"/>
-      <c r="D36" s="103"/>
-      <c r="E36" s="103"/>
-      <c r="F36" s="103"/>
-      <c r="G36" s="103"/>
-      <c r="H36" s="103"/>
-      <c r="I36" s="104"/>
+      <c r="B36" s="137"/>
+      <c r="C36" s="115"/>
+      <c r="D36" s="115"/>
+      <c r="E36" s="115"/>
+      <c r="F36" s="115"/>
+      <c r="G36" s="115"/>
+      <c r="H36" s="115"/>
+      <c r="I36" s="116"/>
       <c r="J36" s="70"/>
       <c r="K36" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L36" s="72"/>
-      <c r="M36" s="98"/>
-      <c r="N36" s="99"/>
+      <c r="M36" s="163"/>
+      <c r="N36" s="127"/>
     </row>
     <row r="37" spans="1:14" ht="13.5" customHeight="1">
       <c r="A37" s="69"/>
-      <c r="B37" s="124"/>
-      <c r="C37" s="103"/>
-      <c r="D37" s="103"/>
-      <c r="E37" s="103"/>
-      <c r="F37" s="103"/>
-      <c r="G37" s="103"/>
-      <c r="H37" s="103"/>
-      <c r="I37" s="104"/>
+      <c r="B37" s="137"/>
+      <c r="C37" s="115"/>
+      <c r="D37" s="115"/>
+      <c r="E37" s="115"/>
+      <c r="F37" s="115"/>
+      <c r="G37" s="115"/>
+      <c r="H37" s="115"/>
+      <c r="I37" s="116"/>
       <c r="J37" s="70"/>
       <c r="K37" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L37" s="72"/>
-      <c r="M37" s="98"/>
-      <c r="N37" s="99"/>
+      <c r="M37" s="163"/>
+      <c r="N37" s="127"/>
     </row>
     <row r="38" spans="1:14" ht="13.5" customHeight="1">
       <c r="A38" s="69"/>
-      <c r="B38" s="124"/>
-      <c r="C38" s="103"/>
-      <c r="D38" s="103"/>
-      <c r="E38" s="103"/>
-      <c r="F38" s="103"/>
-      <c r="G38" s="103"/>
-      <c r="H38" s="103"/>
-      <c r="I38" s="104"/>
+      <c r="B38" s="137"/>
+      <c r="C38" s="115"/>
+      <c r="D38" s="115"/>
+      <c r="E38" s="115"/>
+      <c r="F38" s="115"/>
+      <c r="G38" s="115"/>
+      <c r="H38" s="115"/>
+      <c r="I38" s="116"/>
       <c r="J38" s="70"/>
       <c r="K38" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L38" s="72"/>
-      <c r="M38" s="98"/>
-      <c r="N38" s="99"/>
+      <c r="M38" s="163"/>
+      <c r="N38" s="127"/>
     </row>
     <row r="39" spans="1:14" ht="13.5" customHeight="1">
       <c r="A39" s="69"/>
-      <c r="B39" s="124"/>
-      <c r="C39" s="103"/>
-      <c r="D39" s="103"/>
-      <c r="E39" s="103"/>
-      <c r="F39" s="103"/>
-      <c r="G39" s="103"/>
-      <c r="H39" s="103"/>
-      <c r="I39" s="104"/>
+      <c r="B39" s="137"/>
+      <c r="C39" s="115"/>
+      <c r="D39" s="115"/>
+      <c r="E39" s="115"/>
+      <c r="F39" s="115"/>
+      <c r="G39" s="115"/>
+      <c r="H39" s="115"/>
+      <c r="I39" s="116"/>
       <c r="J39" s="70"/>
       <c r="K39" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L39" s="72"/>
-      <c r="M39" s="98"/>
-      <c r="N39" s="99"/>
+      <c r="M39" s="163"/>
+      <c r="N39" s="127"/>
     </row>
     <row r="40" spans="1:14" ht="13.5" customHeight="1">
       <c r="A40" s="69"/>
-      <c r="B40" s="124"/>
-      <c r="C40" s="103"/>
-      <c r="D40" s="103"/>
-      <c r="E40" s="103"/>
-      <c r="F40" s="103"/>
-      <c r="G40" s="103"/>
-      <c r="H40" s="103"/>
-      <c r="I40" s="104"/>
+      <c r="B40" s="137"/>
+      <c r="C40" s="115"/>
+      <c r="D40" s="115"/>
+      <c r="E40" s="115"/>
+      <c r="F40" s="115"/>
+      <c r="G40" s="115"/>
+      <c r="H40" s="115"/>
+      <c r="I40" s="116"/>
       <c r="J40" s="70"/>
       <c r="K40" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L40" s="72"/>
-      <c r="M40" s="98"/>
-      <c r="N40" s="99"/>
+      <c r="M40" s="163"/>
+      <c r="N40" s="127"/>
     </row>
     <row r="41" spans="1:14" ht="13.5" customHeight="1">
       <c r="A41" s="74"/>
-      <c r="B41" s="125"/>
-      <c r="C41" s="126"/>
-      <c r="D41" s="126"/>
-      <c r="E41" s="126"/>
-      <c r="F41" s="126"/>
-      <c r="G41" s="126"/>
-      <c r="H41" s="126"/>
-      <c r="I41" s="127"/>
+      <c r="B41" s="138"/>
+      <c r="C41" s="139"/>
+      <c r="D41" s="139"/>
+      <c r="E41" s="139"/>
+      <c r="F41" s="139"/>
+      <c r="G41" s="139"/>
+      <c r="H41" s="139"/>
+      <c r="I41" s="140"/>
       <c r="J41" s="75"/>
       <c r="K41" s="76">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L41" s="77"/>
-      <c r="M41" s="110"/>
-      <c r="N41" s="111"/>
+      <c r="M41" s="166"/>
+      <c r="N41" s="167"/>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
       <c r="A42" s="78"/>

</xml_diff>

<commit_message>
corrección en formato de la plantilla excel en pie de pagina
</commit_message>
<xml_diff>
--- a/netlify/functions/plantilla.xlsx
+++ b/netlify/functions/plantilla.xlsx
@@ -2945,7 +2945,6 @@
       <c r="G26" s="141"/>
       <c r="H26" s="141"/>
       <c r="I26" s="141"/>
-      <c r="J26" s="38"/>
       <c r="K26" s="45"/>
       <c r="L26" s="46"/>
       <c r="M26" s="46"/>
@@ -3367,8 +3366,8 @@
   <pageMargins left="0.86614173228346458" right="0.39370078740157483" top="1.1811023622047245" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
-    <oddHeader>&amp;C* Formulario de Solicitud y Aprobacion de Pago *</oddHeader>
-    <oddFooter>&amp;R00-024βэηяμ</oddFooter>
+    <oddHeader>&amp;C
+* Formulario de Solicitud y Aprobacion de Pago *</oddHeader>
   </headerFooter>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>